<commit_message>
T46 hit-zone overlay (axe circle, hurt rects), axe hit radius slider, sliding stick anchor
- panel UKAZ ZONY ZASAHU draws axe circle and enemy/hero hurt rectangles
- axe hit radius live from panel
- left stick centre follows the thumb past full-speed distance (free_move_anchor_slides)
- panel list: the two "posun palca" sliders stay visible by default

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JWzSYD8PFy4XvrWkxJFyL4
</commit_message>
<xml_diff>
--- a/PANEL_prvky.xlsx
+++ b/PANEL_prvky.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Panel'!$A$1:$G$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Panel'!$A$1:$G$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H74"/>
+  <dimension ref="A1:H76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1955,12 +1955,12 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Ovladanie: ako daleko treba posunut palec pre plnu rychlost.</t>
+          <t>Ako daleko od stredu paky treba posunut palec pre plnu rychlost (mensie cislo = rychlejsie plna rychlost, kratsia pomala zona).</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -1997,12 +1997,12 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>To iste, vpravo.</t>
+          <t>To iste, vpravo; plati aj pre pohyb hore a dole.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2613,7 +2613,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>UKAZ ZONU UDERU BEZCA</t>
+          <t>UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2623,17 +2623,17 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Nakresli kruh, kam dopadne uder bezca.</t>
+          <t>Nakresli kruh sekery a obdlzniky zasahu nepriatelov a hrdinu.</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>switch|UKAZ ZONU UDERU BEZCA</t>
+          <t>switch|UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
         </is>
       </c>
     </row>
@@ -2655,27 +2655,27 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
+          <t>sekera: polomer zasahu (px)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Poloha zony uderu.</t>
+          <t>Velkost kruhu sekery; sekera zasiahne kazdeho, koho obdlznik sa dotkne kruhu.</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>slider|zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
+          <t>slider|sekera: polomer zasahu (px)</t>
         </is>
       </c>
     </row>
@@ -2692,22 +2692,22 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: vyska dopadu nad nohami bezca (px)</t>
+          <t>UKAZ ZONU UDERU BEZCA</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Poloha zony uderu.</t>
+          <t>Nakresli kruh, kam dopadne uder bezca.</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>slider|zona uderu: vyska dopadu nad nohami bezca (px)</t>
+          <t>switch|UKAZ ZONU UDERU BEZCA</t>
         </is>
       </c>
     </row>
@@ -2739,7 +2739,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
+          <t>zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Velkost zony uderu.</t>
+          <t>Poloha zony uderu.</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>slider|zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
+          <t>slider|zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
         </is>
       </c>
     </row>
@@ -2781,17 +2781,17 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
+          <t>zona uderu: vyska dopadu nad nohami bezca (px)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Casovanie zasahu v animacii.</t>
+          <t>Poloha zony uderu.</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>slider|kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
+          <t>slider|zona uderu: vyska dopadu nad nohami bezca (px)</t>
         </is>
       </c>
     </row>
@@ -2823,17 +2823,17 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
+          <t>zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Vyska zasiahnutelnej casti nepriatela.</t>
+          <t>Velkost zony uderu.</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>slider|aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
+          <t>slider|zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
         </is>
       </c>
     </row>
@@ -2860,32 +2860,32 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>PEVNE TELA (nikto cez nikoho neprejde)</t>
+          <t>kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Zapne pevne nohy postav; nikto cez nikoho neprejde.</t>
+          <t>Casovanie zasahu v animacii.</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>switch|PEVNE TELA (nikto cez nikoho neprejde)</t>
+          <t>slider|kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
         </is>
       </c>
     </row>
@@ -2907,17 +2907,17 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>pevne telo: hlbka nohy (px; 54 = cele telo)</t>
+          <t>aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Hlbka pevneho tela (odladene 30).</t>
+          <t>Vyska zasiahnutelnej casti nepriatela.</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2927,7 +2927,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>slider|pevne telo: hlbka nohy (px; 54 = cele telo)</t>
+          <t>slider|aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
         </is>
       </c>
     </row>
@@ -2944,32 +2944,32 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>pevne telo: sirka nohy (px)</t>
+          <t>PEVNE TELA (nikto cez nikoho neprejde)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Sirka pevneho tela (odladene 60).</t>
+          <t>Zapne pevne nohy postav; nikto cez nikoho neprejde.</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>slider|pevne telo: sirka nohy (px)</t>
+          <t>switch|PEVNE TELA (nikto cez nikoho neprejde)</t>
         </is>
       </c>
     </row>
@@ -2991,17 +2991,17 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
+          <t>pevne telo: hlbka nohy (px; 54 = cele telo)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Stary mak odtlacania; funguje len ked su PEVNE TELA vypnute.</t>
+          <t>Hlbka pevneho tela (odladene 30).</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>slider|ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
+          <t>slider|pevne telo: hlbka nohy (px; 54 = cele telo)</t>
         </is>
       </c>
     </row>
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3033,27 +3033,27 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>bezec odhodi hrdinu (px)</t>
+          <t>pevne telo: sirka nohy (px)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu po zasahu bezca.</t>
+          <t>Sirka pevneho tela (odladene 60).</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>slider|bezec odhodi hrdinu (px)</t>
+          <t>slider|pevne telo: sirka nohy (px)</t>
         </is>
       </c>
     </row>
@@ -3065,7 +3065,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3075,27 +3075,27 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>strela strelca odhodi hrdinu (px)</t>
+          <t>ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu po zasahu strely.</t>
+          <t>Stary mak odtlacania; funguje len ked su PEVNE TELA vypnute.</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>slider|strela strelca odhodi hrdinu (px)</t>
+          <t>slider|ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
         </is>
       </c>
     </row>
@@ -3117,17 +3117,17 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>sekera odhodi nepriatela (px)</t>
+          <t>bezec odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>90.0</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia nepriatela po zasahu sekery.</t>
+          <t>Dlzka odhodenia hrdinu po zasahu bezca.</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3137,7 +3137,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>slider|sekera odhodi nepriatela (px)</t>
+          <t>slider|bezec odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -3159,17 +3159,17 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>vybuch kotla odhodi hrdinu (px)</t>
+          <t>strela strelca odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>140.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu pri vybuchu kotla.</t>
+          <t>Dlzka odhodenia hrdinu po zasahu strely.</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3179,7 +3179,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>slider|vybuch kotla odhodi hrdinu (px)</t>
+          <t>slider|strela strelca odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -3201,27 +3201,27 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>odhodenie: ako dlho trva (s)</t>
+          <t>sekera odhodi nepriatela (px)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Trvanie odhodenia (odladene 0,4).</t>
+          <t>Dlzka odhodenia nepriatela po zasahu sekery.</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>slider|odhodenie: ako dlho trva (s)</t>
+          <t>slider|sekera odhodi nepriatela (px)</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>ODHODENIE PO ZASAHU</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3243,17 +3243,17 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+          <t>vybuch kotla odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>140.0</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Zivoty nad postavami.</t>
+          <t>Dlzka odhodenia hrdinu pri vybuchu kotla.</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>slider|srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+          <t>slider|vybuch kotla odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>ODHODENIE PO ZASAHU</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3285,17 +3285,17 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>tien pod postavami: sila (0 = vypnuty)</t>
+          <t>odhodenie: ako dlho trva (s)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Sila tiena (odladene 0,3).</t>
+          <t>Trvanie odhodenia (odladene 0,4).</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3305,7 +3305,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>slider|tien pod postavami: sila (0 = vypnuty)</t>
+          <t>slider|odhodenie: ako dlho trva (s)</t>
         </is>
       </c>
     </row>
@@ -3327,27 +3327,27 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>tien pod postavami: velkost (x)</t>
+          <t>srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Velkost tiena (odladene 1).</t>
+          <t>Zivoty nad postavami.</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>slider|tien pod postavami: velkost (x)</t>
+          <t>slider|srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
         </is>
       </c>
     </row>
@@ -3359,7 +3359,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>SRDIECKA A TIENE</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3369,17 +3369,17 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>sirka</t>
+          <t>tien pod postavami: sila (0 = vypnuty)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Sirka zony pre lavy palec.</t>
+          <t>Sila tiena (odladene 0,3).</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -3389,7 +3389,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>slider|sirka</t>
+          <t>slider|tien pod postavami: sila (0 = vypnuty)</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>SRDIECKA A TIENE</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3411,17 +3411,17 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>kolko zospodu patri miereniu</t>
+          <t>tien pod postavami: velkost (x)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Spodna cast zony patri miereniu.</t>
+          <t>Velkost tiena (odladene 1).</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3431,7 +3431,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>slider|kolko zospodu patri miereniu</t>
+          <t>slider|tien pod postavami: velkost (x)</t>
         </is>
       </c>
     </row>
@@ -3448,22 +3448,22 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>MIERIT OD POSTAVY</t>
+          <t>sirka</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Mierenie zacina od postavy.</t>
+          <t>Sirka zony pre lavy palec.</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3473,7 +3473,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>switch|MIERIT OD POSTAVY</t>
+          <t>slider|sirka</t>
         </is>
       </c>
     </row>
@@ -3490,22 +3490,22 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>VOLNY POHYB (bez skoku)</t>
+          <t>kolko zospodu patri miereniu</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>0.16</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Hrdina nechodi skokom k prstu.</t>
+          <t>Spodna cast zony patri miereniu.</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>switch|VOLNY POHYB (bez skoku)</t>
+          <t>slider|kolko zospodu patri miereniu</t>
         </is>
       </c>
     </row>
@@ -3537,33 +3537,117 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
+          <t>MIERIT OD POSTAVY</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>ZAP</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Mierenie zacina od postavy.</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>switch|MIERIT OD POSTAVY</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>S74</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>switch</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>VOLNY POHYB (bez skoku)</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ZAP</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Hrdina nechodi skokom k prstu.</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>switch|VOLNY POHYB (bez skoku)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>S75</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>switch</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
           <t>POHYB KOPIRUJE PALEC</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
+      <c r="E76" t="inlineStr">
         <is>
           <t>VYP</t>
         </is>
       </c>
-      <c r="F74" s="2" t="inlineStr">
+      <c r="F76" s="2" t="inlineStr">
         <is>
           <t>Hrdina kopiruje pohyb palca.</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
         <is>
           <t>switch|POHYB KOPIRUJE PALEC</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G74"/>
-  <conditionalFormatting sqref="G2:G74">
+  <autoFilter ref="A1:G76"/>
+  <conditionalFormatting sqref="G2:G76">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"A"</formula>
     </cfRule>
@@ -3572,7 +3656,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"A,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Package 1 step A: hit-stop, white flash, shake, camera kick, axe-hit buzz with panel switches (A1 A2 A3 A4 E1 P1)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PANEL_prvky.xlsx
+++ b/PANEL_prvky.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Panel'!$A$1:$G$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Panel'!$A$1:$G$86</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H76"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1567,17 +1567,17 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>HUDBA</t>
+          <t>ZASTAVENIE PRI ZASAHU</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Zapne/vypne hudbu.</t>
+          <t>Pri zasahu tvojej zbrane sa hra na okamih zastavi (pocit tazkeho uderu).</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>switch|HUDBA</t>
+          <t>switch|ZASTAVENIE PRI ZASAHU</t>
         </is>
       </c>
     </row>
@@ -1609,27 +1609,27 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>hlasitost hudby (dB)</t>
+          <t>zastavenie pri zasahu (ms)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Hlasitost hudby.</t>
+          <t>Ako dlho trva zastavenie pri zasahu (pri zabiti dlhsie).</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>slider|hlasitost hudby (dB)</t>
+          <t>slider|zastavenie pri zasahu (ms)</t>
         </is>
       </c>
     </row>
@@ -1651,17 +1651,17 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>ZMRAZIT SVET (hybe sa len hrdina)</t>
+          <t>BIELY ZABLESK</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Zastavi nepriatelov, kotly a ich strely; hybe sa len hrdina.</t>
+          <t>Zasiahnuty nepriatel na chvilu cely zbeli.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>switch|ZMRAZIT SVET (hybe sa len hrdina)</t>
+          <t>switch|BIELY ZABLESK</t>
         </is>
       </c>
     </row>
@@ -1688,22 +1688,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT BEZCOV</t>
+          <t>dlzka bieleho zablesku (ms)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat bezci.</t>
+          <t>Ako dlho je nepriatel biely.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1713,7 +1713,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>switch|VYPNUT BEZCOV</t>
+          <t>slider|dlzka bieleho zablesku (ms)</t>
         </is>
       </c>
     </row>
@@ -1735,17 +1735,17 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT STRELCOV</t>
+          <t>TRASENIE OBRAZU PRI ZASAHU</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat strelci.</t>
+          <t>Obrazovka sa zatrasie pri zasahu a zabiti sekerou.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>switch|VYPNUT STRELCOV</t>
+          <t>switch|TRASENIE OBRAZU PRI ZASAHU</t>
         </is>
       </c>
     </row>
@@ -1772,22 +1772,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT TUCNAKOV</t>
+          <t>sila trasenia pri zasahu</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat tucniaci.</t>
+          <t>Nasobok sily trasenia (1.0 = zakladna).</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>switch|VYPNUT TUCNAKOV</t>
+          <t>slider|sila trasenia pri zasahu</t>
         </is>
       </c>
     </row>
@@ -1814,22 +1814,22 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>kolko bezcov naraz (test)</t>
+          <t>KOPNUTIE KAMERY</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Kolko bezcov je naraz v hre.</t>
+          <t>Kamera sa na okamih trhne v smere letu seker/strely.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>slider|kolko bezcov naraz (test)</t>
+          <t>switch|KOPNUTIE KAMERY</t>
         </is>
       </c>
     </row>
@@ -1861,17 +1861,17 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>kolko strelcov naraz (test)</t>
+          <t>sila kopnutia kamery</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Kolko strelcov je naraz v hre.</t>
+          <t>Nasobok sily kopnutia (1.0 = zakladna).</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1881,7 +1881,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>slider|kolko strelcov naraz (test)</t>
+          <t>slider|sila kopnutia kamery</t>
         </is>
       </c>
     </row>
@@ -1898,22 +1898,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>kolko tucnakov naraz (test)</t>
+          <t>VIBRACIA PRI MOJOM ZASAHU</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Kolko tucniakov je naraz v hre.</t>
+          <t>Kratke zavibrovanie telefonu, ked tvoja zbran zasiahne nepriatela.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>slider|kolko tucnakov naraz (test)</t>
+          <t>switch|VIBRACIA PRI MOJOM ZASAHU</t>
         </is>
       </c>
     </row>
@@ -1935,7 +1935,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>POHYB</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1945,17 +1945,17 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>posun palca pre plnu rychlost vlavo</t>
+          <t>dlzka vibracie pri mojom zasahu (ms)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Ako daleko od stredu paky treba posunut palec pre plnu rychlost (mensie cislo = rychlejsie plna rychlost, kratsia pomala zona).</t>
+          <t>Dlzka vibracie pri tvojom zasahu.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>slider|posun palca pre plnu rychlost vlavo</t>
+          <t>slider|dlzka vibracie pri mojom zasahu (ms)</t>
         </is>
       </c>
     </row>
@@ -1977,27 +1977,27 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>POHYB</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>posun palca pre plnu rychlost vpravo</t>
+          <t>HUDBA</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>15.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>To iste, vpravo; plati aj pre pohyb hore a dole.</t>
+          <t>Zapne/vypne hudbu.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>slider|posun palca pre plnu rychlost vpravo</t>
+          <t>switch|HUDBA</t>
         </is>
       </c>
     </row>
@@ -2019,7 +2019,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>POHYB</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2029,27 +2029,27 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>o kolko pomalsi je pohyb hore-dole</t>
+          <t>hlasitost hudby (dB)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>1 = hore/dole rovnako rychlo ako do stran; menej = pomalsie.</t>
+          <t>Hlasitost hudby.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>slider|o kolko pomalsi je pohyb hore-dole</t>
+          <t>slider|hlasitost hudby (dB)</t>
         </is>
       </c>
     </row>
@@ -2061,37 +2061,37 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>ako blizko k postave prestane mierit</t>
+          <t>ZMRAZIT SVET (hybe sa len hrdina)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Mierenie sa vypne, ked je palec blizko postavy.</t>
+          <t>Zastavi nepriatelov, kotly a ich strely; hybe sa len hrdina.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>slider|ako blizko k postave prestane mierit</t>
+          <t>switch|ZMRAZIT SVET (hybe sa len hrdina)</t>
         </is>
       </c>
     </row>
@@ -2103,27 +2103,27 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>rychlost postavy</t>
+          <t>VYPNUT BEZCOV</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti hrdinu.</t>
+          <t>Nebudu sa objavovat bezci.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>slider|rychlost postavy</t>
+          <t>switch|VYPNUT BEZCOV</t>
         </is>
       </c>
     </row>
@@ -2145,37 +2145,37 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>pohyb pocas hodu (0 = stoji)</t>
+          <t>VYPNUT STRELCOV</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Ako rychlo sa hrdina hybe pocas hodu.</t>
+          <t>Nebudu sa objavovat strelci.</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>slider|pohyb pocas hodu (0 = stoji)</t>
+          <t>switch|VYPNUT STRELCOV</t>
         </is>
       </c>
     </row>
@@ -2187,37 +2187,37 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>rychlost zamachu pri hode (1 = povodna)</t>
+          <t>VYPNUT TUCNAKOV</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Rychlost animacie hodu.</t>
+          <t>Nebudu sa objavovat tucniaci.</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>slider|rychlost zamachu pri hode (1 = povodna)</t>
+          <t>switch|VYPNUT TUCNAKOV</t>
         </is>
       </c>
     </row>
@@ -2229,37 +2229,37 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>HRDINA 2x (vypnute = 1x)</t>
+          <t>kolko bezcov naraz (test)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Velkost hrdinu.</t>
+          <t>Kolko bezcov je naraz v hre.</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>switch|HRDINA 2x (vypnute = 1x)</t>
+          <t>slider|kolko bezcov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -2271,27 +2271,27 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>SEKERA (vypnute = gulky)</t>
+          <t>kolko strelcov naraz (test)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Prepina zbran: sekera alebo gulky.</t>
+          <t>Kolko strelcov je naraz v hre.</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>switch|SEKERA (vypnute = gulky)</t>
+          <t>slider|kolko strelcov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2313,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2323,17 +2323,17 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>dosah sekery</t>
+          <t>kolko tucnakov naraz (test)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>350.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Ako daleko sekera doletí.</t>
+          <t>Kolko tucniakov je naraz v hre.</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2343,7 +2343,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>slider|dosah sekery</t>
+          <t>slider|kolko tucnakov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -2355,7 +2355,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>POHYB</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2365,17 +2365,17 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>rychlost sekery</t>
+          <t>posun palca pre plnu rychlost vlavo</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>650.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Rychlost sekery smerom k cielu (spat je 1,5x).</t>
+          <t>Ako daleko od stredu paky treba posunut palec pre plnu rychlost (mensie cislo = rychlejsie plna rychlost, kratsia pomala zona).</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>slider|rychlost sekery</t>
+          <t>slider|posun palca pre plnu rychlost vlavo</t>
         </is>
       </c>
     </row>
@@ -2397,23 +2397,27 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>POHYB</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>NOVE SUDY (postavi ich pred hrdinu)</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr"/>
+          <t>posun palca pre plnu rychlost vpravo</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>15.0</t>
+        </is>
+      </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Tlacidlo: znova postavi sudy.</t>
+          <t>To iste, vpravo; plati aj pre pohyb hore a dole.</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2423,7 +2427,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>button|NOVE SUDY (postavi ich pred hrdinu)</t>
+          <t>slider|posun palca pre plnu rychlost vpravo</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2439,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>POHYB</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2445,27 +2449,27 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>aky vysoky kus tela hraca sa da trafit (0-1)</t>
+          <t>o kolko pomalsi je pohyb hore-dole</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Vyska zasiahnutelnej casti hrdinu.</t>
+          <t>1 = hore/dole rovnako rychlo ako do stran; menej = pomalsie.</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>slider|aky vysoky kus tela hraca sa da trafit (0-1)</t>
+          <t>slider|o kolko pomalsi je pohyb hore-dole</t>
         </is>
       </c>
     </row>
@@ -2477,7 +2481,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2487,27 +2491,27 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>rychlost bezcov</t>
+          <t>ako blizko k postave prestane mierit</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti bezcov.</t>
+          <t>Mierenie sa vypne, ked je palec blizko postavy.</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>slider|rychlost bezcov</t>
+          <t>slider|ako blizko k postave prestane mierit</t>
         </is>
       </c>
     </row>
@@ -2519,7 +2523,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2529,7 +2533,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>rychlost strelcov</t>
+          <t>rychlost postavy</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2539,7 +2543,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti strelcov.</t>
+          <t>Nasobok rychlosti hrdinu.</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2549,7 +2553,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>slider|rychlost strelcov</t>
+          <t>slider|rychlost postavy</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2565,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2571,17 +2575,17 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>na aku vzdialenost si bezec vsimne hraca (px)</t>
+          <t>pohyb pocas hodu (0 = stoji)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>640.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Dosah, od ktoreho bezec zacne prenasledovat.</t>
+          <t>Ako rychlo sa hrdina hybe pocas hodu.</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2591,7 +2595,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>slider|na aku vzdialenost si bezec vsimne hraca (px)</t>
+          <t>slider|pohyb pocas hodu (0 = stoji)</t>
         </is>
       </c>
     </row>
@@ -2603,37 +2607,37 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
+          <t>rychlost zamachu pri hode (1 = povodna)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Nakresli kruh sekery a obdlzniky zasahu nepriatelov a hrdinu.</t>
+          <t>Rychlost animacie hodu.</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>switch|UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
+          <t>slider|rychlost zamachu pri hode (1 = povodna)</t>
         </is>
       </c>
     </row>
@@ -2645,37 +2649,37 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>sekera: polomer zasahu (px)</t>
+          <t>HRDINA 2x (vypnute = 1x)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Velkost kruhu sekery; sekera zasiahne kazdeho, koho obdlznik sa dotkne kruhu.</t>
+          <t>Velkost hrdinu.</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>slider|sekera: polomer zasahu (px)</t>
+          <t>switch|HRDINA 2x (vypnute = 1x)</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2691,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2697,27 +2701,27 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>UKAZ ZONU UDERU BEZCA</t>
+          <t>SEKERA (vypnute = gulky)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Nakresli kruh, kam dopadne uder bezca.</t>
+          <t>Prepina zbran: sekera alebo gulky.</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>switch|UKAZ ZONU UDERU BEZCA</t>
+          <t>switch|SEKERA (vypnute = gulky)</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2733,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2739,27 +2743,27 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
+          <t>dosah sekery</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>350.0</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Poloha zony uderu.</t>
+          <t>Ako daleko sekera doletí.</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>slider|zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
+          <t>slider|dosah sekery</t>
         </is>
       </c>
     </row>
@@ -2771,7 +2775,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2781,27 +2785,27 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: vyska dopadu nad nohami bezca (px)</t>
+          <t>rychlost sekery</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>650.0</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Poloha zony uderu.</t>
+          <t>Rychlost sekery smerom k cielu (spat je 1,5x).</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>slider|zona uderu: vyska dopadu nad nohami bezca (px)</t>
+          <t>slider|rychlost sekery</t>
         </is>
       </c>
     </row>
@@ -2813,37 +2817,33 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>button</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>40.0</t>
-        </is>
-      </c>
+          <t>NOVE SUDY (postavi ich pred hrdinu)</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Velkost zony uderu.</t>
+          <t>Tlacidlo: znova postavi sudy.</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>slider|zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
+          <t>button|NOVE SUDY (postavi ich pred hrdinu)</t>
         </is>
       </c>
     </row>
@@ -2855,7 +2855,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2865,17 +2865,17 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
+          <t>aky vysoky kus tela hraca sa da trafit (0-1)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Casovanie zasahu v animacii.</t>
+          <t>Vyska zasiahnutelnej casti hrdinu.</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>slider|kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
+          <t>slider|aky vysoky kus tela hraca sa da trafit (0-1)</t>
         </is>
       </c>
     </row>
@@ -2907,27 +2907,27 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
+          <t>rychlost bezcov</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Vyska zasiahnutelnej casti nepriatela.</t>
+          <t>Nasobok rychlosti bezcov.</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>slider|aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
+          <t>slider|rychlost bezcov</t>
         </is>
       </c>
     </row>
@@ -2944,22 +2944,22 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>PEVNE TELA (nikto cez nikoho neprejde)</t>
+          <t>rychlost strelcov</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Zapne pevne nohy postav; nikto cez nikoho neprejde.</t>
+          <t>Nasobok rychlosti strelcov.</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>switch|PEVNE TELA (nikto cez nikoho neprejde)</t>
+          <t>slider|rychlost strelcov</t>
         </is>
       </c>
     </row>
@@ -2991,17 +2991,17 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>pevne telo: hlbka nohy (px; 54 = cele telo)</t>
+          <t>na aku vzdialenost si bezec vsimne hraca (px)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>640.0</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Hlbka pevneho tela (odladene 30).</t>
+          <t>Dosah, od ktoreho bezec zacne prenasledovat.</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>slider|pevne telo: hlbka nohy (px; 54 = cele telo)</t>
+          <t>slider|na aku vzdialenost si bezec vsimne hraca (px)</t>
         </is>
       </c>
     </row>
@@ -3028,32 +3028,32 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>pevne telo: sirka nohy (px)</t>
+          <t>UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Sirka pevneho tela (odladene 60).</t>
+          <t>Nakresli kruh sekery a obdlzniky zasahu nepriatelov a hrdinu.</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>slider|pevne telo: sirka nohy (px)</t>
+          <t>switch|UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
         </is>
       </c>
     </row>
@@ -3075,27 +3075,27 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
+          <t>sekera: polomer zasahu (px)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Stary mak odtlacania; funguje len ked su PEVNE TELA vypnute.</t>
+          <t>Velkost kruhu sekery; sekera zasiahne kazdeho, koho obdlznik sa dotkne kruhu.</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>slider|ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
+          <t>slider|sekera: polomer zasahu (px)</t>
         </is>
       </c>
     </row>
@@ -3107,37 +3107,37 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>bezec odhodi hrdinu (px)</t>
+          <t>UKAZ ZONU UDERU BEZCA</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu po zasahu bezca.</t>
+          <t>Nakresli kruh, kam dopadne uder bezca.</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>slider|bezec odhodi hrdinu (px)</t>
+          <t>switch|UKAZ ZONU UDERU BEZCA</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3159,27 +3159,27 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>strela strelca odhodi hrdinu (px)</t>
+          <t>zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu po zasahu strely.</t>
+          <t>Poloha zony uderu.</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>slider|strela strelca odhodi hrdinu (px)</t>
+          <t>slider|zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3201,27 +3201,27 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>sekera odhodi nepriatela (px)</t>
+          <t>zona uderu: vyska dopadu nad nohami bezca (px)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia nepriatela po zasahu sekery.</t>
+          <t>Poloha zony uderu.</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>slider|sekera odhodi nepriatela (px)</t>
+          <t>slider|zona uderu: vyska dopadu nad nohami bezca (px)</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3243,27 +3243,27 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>vybuch kotla odhodi hrdinu (px)</t>
+          <t>zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>140.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu pri vybuchu kotla.</t>
+          <t>Velkost zony uderu.</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>slider|vybuch kotla odhodi hrdinu (px)</t>
+          <t>slider|zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3285,17 +3285,17 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>odhodenie: ako dlho trva (s)</t>
+          <t>kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Trvanie odhodenia (odladene 0,4).</t>
+          <t>Casovanie zasahu v animacii.</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3305,7 +3305,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>slider|odhodenie: ako dlho trva (s)</t>
+          <t>slider|kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
         </is>
       </c>
     </row>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3327,27 +3327,27 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+          <t>aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Zivoty nad postavami.</t>
+          <t>Vyska zasiahnutelnej casti nepriatela.</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>slider|srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+          <t>slider|aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
         </is>
       </c>
     </row>
@@ -3359,37 +3359,37 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>tien pod postavami: sila (0 = vypnuty)</t>
+          <t>PEVNE TELA (nikto cez nikoho neprejde)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Sila tiena (odladene 0,3).</t>
+          <t>Zapne pevne nohy postav; nikto cez nikoho neprejde.</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>slider|tien pod postavami: sila (0 = vypnuty)</t>
+          <t>switch|PEVNE TELA (nikto cez nikoho neprejde)</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3411,17 +3411,17 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>tien pod postavami: velkost (x)</t>
+          <t>pevne telo: hlbka nohy (px; 54 = cele telo)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Velkost tiena (odladene 1).</t>
+          <t>Hlbka pevneho tela (odladene 30).</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3431,7 +3431,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>slider|tien pod postavami: velkost (x)</t>
+          <t>slider|pevne telo: hlbka nohy (px; 54 = cele telo)</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3453,17 +3453,17 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>sirka</t>
+          <t>pevne telo: sirka nohy (px)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Sirka zony pre lavy palec.</t>
+          <t>Sirka pevneho tela (odladene 60).</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3473,7 +3473,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>slider|sirka</t>
+          <t>slider|pevne telo: sirka nohy (px)</t>
         </is>
       </c>
     </row>
@@ -3485,7 +3485,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3495,17 +3495,17 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>kolko zospodu patri miereniu</t>
+          <t>ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Spodna cast zony patri miereniu.</t>
+          <t>Stary mak odtlacania; funguje len ked su PEVNE TELA vypnute.</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>slider|kolko zospodu patri miereniu</t>
+          <t>slider|ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
         </is>
       </c>
     </row>
@@ -3527,37 +3527,37 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>ODHODENIE PO ZASAHU</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>MIERIT OD POSTAVY</t>
+          <t>bezec odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>90.0</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Mierenie zacina od postavy.</t>
+          <t>Dlzka odhodenia hrdinu po zasahu bezca.</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>switch|MIERIT OD POSTAVY</t>
+          <t>slider|bezec odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -3569,37 +3569,37 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>ODHODENIE PO ZASAHU</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>VOLNY POHYB (bez skoku)</t>
+          <t>strela strelca odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Hrdina nechodi skokom k prstu.</t>
+          <t>Dlzka odhodenia hrdinu po zasahu strely.</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>switch|VOLNY POHYB (bez skoku)</t>
+          <t>slider|strela strelca odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -3611,43 +3611,463 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
+          <t>ODHODENIE PO ZASAHU</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>sekera odhodi nepriatela (px)</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>70.0</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Dlzka odhodenia nepriatela po zasahu sekery.</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>slider|sekera odhodi nepriatela (px)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>S76</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>ODHODENIE PO ZASAHU</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>vybuch kotla odhodi hrdinu (px)</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>140.0</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Dlzka odhodenia hrdinu pri vybuchu kotla.</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>slider|vybuch kotla odhodi hrdinu (px)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>S77</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>ODHODENIE PO ZASAHU</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>odhodenie: ako dlho trva (s)</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>Trvanie odhodenia (odladene 0,4).</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>slider|odhodenie: ako dlho trva (s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>S78</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>SRDIECKA A TIENE</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Zivoty nad postavami.</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>slider|srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>S79</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>SRDIECKA A TIENE</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>tien pod postavami: sila (0 = vypnuty)</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Sila tiena (odladene 0,3).</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>slider|tien pod postavami: sila (0 = vypnuty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>S80</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>SRDIECKA A TIENE</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>tien pod postavami: velkost (x)</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>Velkost tiena (odladene 1).</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>slider|tien pod postavami: velkost (x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>S81</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
           <t>ZONA PRE LAVY PALEC</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>sirka</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>Sirka zony pre lavy palec.</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>slider|sirka</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>S82</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>kolko zospodu patri miereniu</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>0.16</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>Spodna cast zony patri miereniu.</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>slider|kolko zospodu patri miereniu</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>S83</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
         <is>
           <t>switch</t>
         </is>
       </c>
-      <c r="D76" s="2" t="inlineStr">
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>MIERIT OD POSTAVY</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>ZAP</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>Mierenie zacina od postavy.</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>switch|MIERIT OD POSTAVY</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>S84</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>switch</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>VOLNY POHYB (bez skoku)</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>ZAP</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>Hrdina nechodi skokom k prstu.</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>switch|VOLNY POHYB (bez skoku)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>S85</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>switch</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
         <is>
           <t>POHYB KOPIRUJE PALEC</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
+      <c r="E86" t="inlineStr">
         <is>
           <t>VYP</t>
         </is>
       </c>
-      <c r="F76" s="2" t="inlineStr">
+      <c r="F86" s="2" t="inlineStr">
         <is>
           <t>Hrdina kopiruje pohyb palca.</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
         <is>
           <t>switch|POHYB KOPIRUJE PALEC</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G76"/>
-  <conditionalFormatting sqref="G2:G76">
+  <autoFilter ref="A1:G86"/>
+  <conditionalFormatting sqref="G2:G86">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"A"</formula>
     </cfRule>
@@ -3656,7 +4076,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G86" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"A,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Bake phone-test values (hit-stop 30 ms, shake and kick x1.5), longer default axe-hit buzz at full amplitude, vibration test button, note T48 observation
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PANEL_prvky.xlsx
+++ b/PANEL_prvky.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Panel'!$A$1:$G$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Panel'!$A$1:$G$87</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H86"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1950,7 +1950,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -1982,22 +1982,18 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>button</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>HUDBA</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>VYP</t>
-        </is>
-      </c>
+          <t>TEST VIBRACIE (rovnaka ako pri mojom zasahu)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Zapne/vypne hudbu.</t>
+          <t>Tlacidlo: jedna vibracia presne taka, ako pri tvojom zasahu (na zistenie, ci telefon vibruje).</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2007,7 +2003,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>switch|HUDBA</t>
+          <t>button|TEST VIBRACIE (rovnaka ako pri mojom zasahu)</t>
         </is>
       </c>
     </row>
@@ -2024,32 +2020,32 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>hlasitost hudby (dB)</t>
+          <t>HUDBA</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Hlasitost hudby.</t>
+          <t>Zapne/vypne hudbu.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>slider|hlasitost hudby (dB)</t>
+          <t>switch|HUDBA</t>
         </is>
       </c>
     </row>
@@ -2066,32 +2062,32 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>ZMRAZIT SVET (hybe sa len hrdina)</t>
+          <t>hlasitost hudby (dB)</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Zastavi nepriatelov, kotly a ich strely; hybe sa len hrdina.</t>
+          <t>Hlasitost hudby.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>switch|ZMRAZIT SVET (hybe sa len hrdina)</t>
+          <t>slider|hlasitost hudby (dB)</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2109,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT BEZCOV</t>
+          <t>ZMRAZIT SVET (hybe sa len hrdina)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2123,7 +2119,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat bezci.</t>
+          <t>Zastavi nepriatelov, kotly a ich strely; hybe sa len hrdina.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2133,7 +2129,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>switch|VYPNUT BEZCOV</t>
+          <t>switch|ZMRAZIT SVET (hybe sa len hrdina)</t>
         </is>
       </c>
     </row>
@@ -2155,7 +2151,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT STRELCOV</t>
+          <t>VYPNUT BEZCOV</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2165,7 +2161,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat strelci.</t>
+          <t>Nebudu sa objavovat bezci.</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2175,7 +2171,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>switch|VYPNUT STRELCOV</t>
+          <t>switch|VYPNUT BEZCOV</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2193,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT TUCNAKOV</t>
+          <t>VYPNUT STRELCOV</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2207,7 +2203,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat tucniaci.</t>
+          <t>Nebudu sa objavovat strelci.</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2217,7 +2213,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>switch|VYPNUT TUCNAKOV</t>
+          <t>switch|VYPNUT STRELCOV</t>
         </is>
       </c>
     </row>
@@ -2234,22 +2230,22 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>kolko bezcov naraz (test)</t>
+          <t>VYPNUT TUCNAKOV</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Kolko bezcov je naraz v hre.</t>
+          <t>Nebudu sa objavovat tucniaci.</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2259,7 +2255,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>slider|kolko bezcov naraz (test)</t>
+          <t>switch|VYPNUT TUCNAKOV</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2277,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>kolko strelcov naraz (test)</t>
+          <t>kolko bezcov naraz (test)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2291,7 +2287,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Kolko strelcov je naraz v hre.</t>
+          <t>Kolko bezcov je naraz v hre.</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2301,7 +2297,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>slider|kolko strelcov naraz (test)</t>
+          <t>slider|kolko bezcov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -2323,17 +2319,17 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>kolko tucnakov naraz (test)</t>
+          <t>kolko strelcov naraz (test)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Kolko tucniakov je naraz v hre.</t>
+          <t>Kolko strelcov je naraz v hre.</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2343,7 +2339,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>slider|kolko tucnakov naraz (test)</t>
+          <t>slider|kolko strelcov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -2355,7 +2351,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>POHYB</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2365,17 +2361,17 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>posun palca pre plnu rychlost vlavo</t>
+          <t>kolko tucnakov naraz (test)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Ako daleko od stredu paky treba posunut palec pre plnu rychlost (mensie cislo = rychlejsie plna rychlost, kratsia pomala zona).</t>
+          <t>Kolko tucniakov je naraz v hre.</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2385,7 +2381,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>slider|posun palca pre plnu rychlost vlavo</t>
+          <t>slider|kolko tucnakov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -2407,17 +2403,17 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>posun palca pre plnu rychlost vpravo</t>
+          <t>posun palca pre plnu rychlost vlavo</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>15.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>To iste, vpravo; plati aj pre pohyb hore a dole.</t>
+          <t>Ako daleko od stredu paky treba posunut palec pre plnu rychlost (mensie cislo = rychlejsie plna rychlost, kratsia pomala zona).</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2427,7 +2423,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>slider|posun palca pre plnu rychlost vpravo</t>
+          <t>slider|posun palca pre plnu rychlost vlavo</t>
         </is>
       </c>
     </row>
@@ -2449,17 +2445,17 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>o kolko pomalsi je pohyb hore-dole</t>
+          <t>posun palca pre plnu rychlost vpravo</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>1 = hore/dole rovnako rychlo ako do stran; menej = pomalsie.</t>
+          <t>To iste, vpravo; plati aj pre pohyb hore a dole.</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2469,7 +2465,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>slider|o kolko pomalsi je pohyb hore-dole</t>
+          <t>slider|posun palca pre plnu rychlost vpravo</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2477,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>POHYB</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2491,27 +2487,27 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>ako blizko k postave prestane mierit</t>
+          <t>o kolko pomalsi je pohyb hore-dole</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Mierenie sa vypne, ked je palec blizko postavy.</t>
+          <t>1 = hore/dole rovnako rychlo ako do stran; menej = pomalsie.</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>slider|ako blizko k postave prestane mierit</t>
+          <t>slider|o kolko pomalsi je pohyb hore-dole</t>
         </is>
       </c>
     </row>
@@ -2533,27 +2529,27 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>rychlost postavy</t>
+          <t>ako blizko k postave prestane mierit</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti hrdinu.</t>
+          <t>Mierenie sa vypne, ked je palec blizko postavy.</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>slider|rychlost postavy</t>
+          <t>slider|ako blizko k postave prestane mierit</t>
         </is>
       </c>
     </row>
@@ -2575,27 +2571,27 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>pohyb pocas hodu (0 = stoji)</t>
+          <t>rychlost postavy</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Ako rychlo sa hrdina hybe pocas hodu.</t>
+          <t>Nasobok rychlosti hrdinu.</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>slider|pohyb pocas hodu (0 = stoji)</t>
+          <t>slider|rychlost postavy</t>
         </is>
       </c>
     </row>
@@ -2617,17 +2613,17 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>rychlost zamachu pri hode (1 = povodna)</t>
+          <t>pohyb pocas hodu (0 = stoji)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Rychlost animacie hodu.</t>
+          <t>Ako rychlo sa hrdina hybe pocas hodu.</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2637,7 +2633,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>slider|rychlost zamachu pri hode (1 = povodna)</t>
+          <t>slider|pohyb pocas hodu (0 = stoji)</t>
         </is>
       </c>
     </row>
@@ -2654,22 +2650,22 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>HRDINA 2x (vypnute = 1x)</t>
+          <t>rychlost zamachu pri hode (1 = povodna)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Velkost hrdinu.</t>
+          <t>Rychlost animacie hodu.</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2679,7 +2675,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>switch|HRDINA 2x (vypnute = 1x)</t>
+          <t>slider|rychlost zamachu pri hode (1 = povodna)</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2697,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>SEKERA (vypnute = gulky)</t>
+          <t>HRDINA 2x (vypnute = 1x)</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2711,17 +2707,17 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Prepina zbran: sekera alebo gulky.</t>
+          <t>Velkost hrdinu.</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>switch|SEKERA (vypnute = gulky)</t>
+          <t>switch|HRDINA 2x (vypnute = 1x)</t>
         </is>
       </c>
     </row>
@@ -2738,22 +2734,22 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>dosah sekery</t>
+          <t>SEKERA (vypnute = gulky)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>350.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Ako daleko sekera doletí.</t>
+          <t>Prepina zbran: sekera alebo gulky.</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2763,7 +2759,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>slider|dosah sekery</t>
+          <t>switch|SEKERA (vypnute = gulky)</t>
         </is>
       </c>
     </row>
@@ -2785,17 +2781,17 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>rychlost sekery</t>
+          <t>dosah sekery</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>650.0</t>
+          <t>350.0</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Rychlost sekery smerom k cielu (spat je 1,5x).</t>
+          <t>Ako daleko sekera doletí.</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2805,7 +2801,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>slider|rychlost sekery</t>
+          <t>slider|dosah sekery</t>
         </is>
       </c>
     </row>
@@ -2822,18 +2818,22 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>NOVE SUDY (postavi ich pred hrdinu)</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr"/>
+          <t>rychlost sekery</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>650.0</t>
+        </is>
+      </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Tlacidlo: znova postavi sudy.</t>
+          <t>Rychlost sekery smerom k cielu (spat je 1,5x).</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>button|NOVE SUDY (postavi ich pred hrdinu)</t>
+          <t>slider|rychlost sekery</t>
         </is>
       </c>
     </row>
@@ -2860,32 +2860,28 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>button</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>aky vysoky kus tela hraca sa da trafit (0-1)</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>0.72</t>
-        </is>
-      </c>
+          <t>NOVE SUDY (postavi ich pred hrdinu)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Vyska zasiahnutelnej casti hrdinu.</t>
+          <t>Tlacidlo: znova postavi sudy.</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>slider|aky vysoky kus tela hraca sa da trafit (0-1)</t>
+          <t>button|NOVE SUDY (postavi ich pred hrdinu)</t>
         </is>
       </c>
     </row>
@@ -2897,7 +2893,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2907,27 +2903,27 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>rychlost bezcov</t>
+          <t>aky vysoky kus tela hraca sa da trafit (0-1)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti bezcov.</t>
+          <t>Vyska zasiahnutelnej casti hrdinu.</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>slider|rychlost bezcov</t>
+          <t>slider|aky vysoky kus tela hraca sa da trafit (0-1)</t>
         </is>
       </c>
     </row>
@@ -2949,7 +2945,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>rychlost strelcov</t>
+          <t>rychlost bezcov</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2959,7 +2955,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti strelcov.</t>
+          <t>Nasobok rychlosti bezcov.</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2969,7 +2965,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>slider|rychlost strelcov</t>
+          <t>slider|rychlost bezcov</t>
         </is>
       </c>
     </row>
@@ -2991,27 +2987,27 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>na aku vzdialenost si bezec vsimne hraca (px)</t>
+          <t>rychlost strelcov</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>640.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Dosah, od ktoreho bezec zacne prenasledovat.</t>
+          <t>Nasobok rychlosti strelcov.</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>slider|na aku vzdialenost si bezec vsimne hraca (px)</t>
+          <t>slider|rychlost strelcov</t>
         </is>
       </c>
     </row>
@@ -3028,32 +3024,32 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
+          <t>na aku vzdialenost si bezec vsimne hraca (px)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>640.0</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Nakresli kruh sekery a obdlzniky zasahu nepriatelov a hrdinu.</t>
+          <t>Dosah, od ktoreho bezec zacne prenasledovat.</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>switch|UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
+          <t>slider|na aku vzdialenost si bezec vsimne hraca (px)</t>
         </is>
       </c>
     </row>
@@ -3070,22 +3066,22 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>sekera: polomer zasahu (px)</t>
+          <t>UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Velkost kruhu sekery; sekera zasiahne kazdeho, koho obdlznik sa dotkne kruhu.</t>
+          <t>Nakresli kruh sekery a obdlzniky zasahu nepriatelov a hrdinu.</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3095,7 +3091,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>slider|sekera: polomer zasahu (px)</t>
+          <t>switch|UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
         </is>
       </c>
     </row>
@@ -3112,32 +3108,32 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>UKAZ ZONU UDERU BEZCA</t>
+          <t>sekera: polomer zasahu (px)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Nakresli kruh, kam dopadne uder bezca.</t>
+          <t>Velkost kruhu sekery; sekera zasiahne kazdeho, koho obdlznik sa dotkne kruhu.</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>switch|UKAZ ZONU UDERU BEZCA</t>
+          <t>slider|sekera: polomer zasahu (px)</t>
         </is>
       </c>
     </row>
@@ -3154,22 +3150,22 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
+          <t>UKAZ ZONU UDERU BEZCA</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Poloha zony uderu.</t>
+          <t>Nakresli kruh, kam dopadne uder bezca.</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3179,7 +3175,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>slider|zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
+          <t>switch|UKAZ ZONU UDERU BEZCA</t>
         </is>
       </c>
     </row>
@@ -3201,12 +3197,12 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: vyska dopadu nad nohami bezca (px)</t>
+          <t>zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -3221,7 +3217,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>slider|zona uderu: vyska dopadu nad nohami bezca (px)</t>
+          <t>slider|zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
         </is>
       </c>
     </row>
@@ -3243,17 +3239,17 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
+          <t>zona uderu: vyska dopadu nad nohami bezca (px)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Velkost zony uderu.</t>
+          <t>Poloha zony uderu.</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3263,7 +3259,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>slider|zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
+          <t>slider|zona uderu: vyska dopadu nad nohami bezca (px)</t>
         </is>
       </c>
     </row>
@@ -3285,17 +3281,17 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
+          <t>zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Casovanie zasahu v animacii.</t>
+          <t>Velkost zony uderu.</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3305,7 +3301,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>slider|kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
+          <t>slider|zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
         </is>
       </c>
     </row>
@@ -3327,17 +3323,17 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
+          <t>kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Vyska zasiahnutelnej casti nepriatela.</t>
+          <t>Casovanie zasahu v animacii.</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3347,7 +3343,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>slider|aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
+          <t>slider|kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
         </is>
       </c>
     </row>
@@ -3364,32 +3360,32 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>PEVNE TELA (nikto cez nikoho neprejde)</t>
+          <t>aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Zapne pevne nohy postav; nikto cez nikoho neprejde.</t>
+          <t>Vyska zasiahnutelnej casti nepriatela.</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>switch|PEVNE TELA (nikto cez nikoho neprejde)</t>
+          <t>slider|aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
         </is>
       </c>
     </row>
@@ -3406,32 +3402,32 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>pevne telo: hlbka nohy (px; 54 = cele telo)</t>
+          <t>PEVNE TELA (nikto cez nikoho neprejde)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Hlbka pevneho tela (odladene 30).</t>
+          <t>Zapne pevne nohy postav; nikto cez nikoho neprejde.</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>slider|pevne telo: hlbka nohy (px; 54 = cele telo)</t>
+          <t>switch|PEVNE TELA (nikto cez nikoho neprejde)</t>
         </is>
       </c>
     </row>
@@ -3453,17 +3449,17 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>pevne telo: sirka nohy (px)</t>
+          <t>pevne telo: hlbka nohy (px; 54 = cele telo)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Sirka pevneho tela (odladene 60).</t>
+          <t>Hlbka pevneho tela (odladene 30).</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3473,7 +3469,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>slider|pevne telo: sirka nohy (px)</t>
+          <t>slider|pevne telo: hlbka nohy (px; 54 = cele telo)</t>
         </is>
       </c>
     </row>
@@ -3495,17 +3491,17 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
+          <t>pevne telo: sirka nohy (px)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Stary mak odtlacania; funguje len ked su PEVNE TELA vypnute.</t>
+          <t>Sirka pevneho tela (odladene 60).</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3515,7 +3511,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>slider|ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
+          <t>slider|pevne telo: sirka nohy (px)</t>
         </is>
       </c>
     </row>
@@ -3527,7 +3523,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3537,27 +3533,27 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>bezec odhodi hrdinu (px)</t>
+          <t>ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu po zasahu bezca.</t>
+          <t>Stary mak odtlacania; funguje len ked su PEVNE TELA vypnute.</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>slider|bezec odhodi hrdinu (px)</t>
+          <t>slider|ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
         </is>
       </c>
     </row>
@@ -3579,17 +3575,17 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>strela strelca odhodi hrdinu (px)</t>
+          <t>bezec odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>90.0</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu po zasahu strely.</t>
+          <t>Dlzka odhodenia hrdinu po zasahu bezca.</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3599,7 +3595,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>slider|strela strelca odhodi hrdinu (px)</t>
+          <t>slider|bezec odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -3621,17 +3617,17 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>sekera odhodi nepriatela (px)</t>
+          <t>strela strelca odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia nepriatela po zasahu sekery.</t>
+          <t>Dlzka odhodenia hrdinu po zasahu strely.</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3641,7 +3637,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>slider|sekera odhodi nepriatela (px)</t>
+          <t>slider|strela strelca odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -3663,17 +3659,17 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>vybuch kotla odhodi hrdinu (px)</t>
+          <t>sekera odhodi nepriatela (px)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>140.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu pri vybuchu kotla.</t>
+          <t>Dlzka odhodenia nepriatela po zasahu sekery.</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3683,7 +3679,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>slider|vybuch kotla odhodi hrdinu (px)</t>
+          <t>slider|sekera odhodi nepriatela (px)</t>
         </is>
       </c>
     </row>
@@ -3705,27 +3701,27 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>odhodenie: ako dlho trva (s)</t>
+          <t>vybuch kotla odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>140.0</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Trvanie odhodenia (odladene 0,4).</t>
+          <t>Dlzka odhodenia hrdinu pri vybuchu kotla.</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>slider|odhodenie: ako dlho trva (s)</t>
+          <t>slider|vybuch kotla odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -3737,7 +3733,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>ODHODENIE PO ZASAHU</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3747,27 +3743,27 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+          <t>odhodenie: ako dlho trva (s)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Zivoty nad postavami.</t>
+          <t>Trvanie odhodenia (odladene 0,4).</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>slider|srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+          <t>slider|odhodenie: ako dlho trva (s)</t>
         </is>
       </c>
     </row>
@@ -3789,27 +3785,27 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>tien pod postavami: sila (0 = vypnuty)</t>
+          <t>srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Sila tiena (odladene 0,3).</t>
+          <t>Zivoty nad postavami.</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>slider|tien pod postavami: sila (0 = vypnuty)</t>
+          <t>slider|srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
         </is>
       </c>
     </row>
@@ -3831,17 +3827,17 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>tien pod postavami: velkost (x)</t>
+          <t>tien pod postavami: sila (0 = vypnuty)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Velkost tiena (odladene 1).</t>
+          <t>Sila tiena (odladene 0,3).</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -3851,7 +3847,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>slider|tien pod postavami: velkost (x)</t>
+          <t>slider|tien pod postavami: sila (0 = vypnuty)</t>
         </is>
       </c>
     </row>
@@ -3863,7 +3859,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>SRDIECKA A TIENE</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3873,17 +3869,17 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>sirka</t>
+          <t>tien pod postavami: velkost (x)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Sirka zony pre lavy palec.</t>
+          <t>Velkost tiena (odladene 1).</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -3893,7 +3889,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>slider|sirka</t>
+          <t>slider|tien pod postavami: velkost (x)</t>
         </is>
       </c>
     </row>
@@ -3915,17 +3911,17 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>kolko zospodu patri miereniu</t>
+          <t>sirka</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Spodna cast zony patri miereniu.</t>
+          <t>Sirka zony pre lavy palec.</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -3935,7 +3931,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>slider|kolko zospodu patri miereniu</t>
+          <t>slider|sirka</t>
         </is>
       </c>
     </row>
@@ -3952,22 +3948,22 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>MIERIT OD POSTAVY</t>
+          <t>kolko zospodu patri miereniu</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>0.16</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Mierenie zacina od postavy.</t>
+          <t>Spodna cast zony patri miereniu.</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -3977,7 +3973,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>switch|MIERIT OD POSTAVY</t>
+          <t>slider|kolko zospodu patri miereniu</t>
         </is>
       </c>
     </row>
@@ -3999,7 +3995,7 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>VOLNY POHYB (bez skoku)</t>
+          <t>MIERIT OD POSTAVY</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4009,7 +4005,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Hrdina nechodi skokom k prstu.</t>
+          <t>Mierenie zacina od postavy.</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -4019,7 +4015,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>switch|VOLNY POHYB (bez skoku)</t>
+          <t>switch|MIERIT OD POSTAVY</t>
         </is>
       </c>
     </row>
@@ -4041,33 +4037,75 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
+          <t>VOLNY POHYB (bez skoku)</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>ZAP</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Hrdina nechodi skokom k prstu.</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>switch|VOLNY POHYB (bez skoku)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>S86</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>switch</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
           <t>POHYB KOPIRUJE PALEC</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
+      <c r="E87" t="inlineStr">
         <is>
           <t>VYP</t>
         </is>
       </c>
-      <c r="F86" s="2" t="inlineStr">
+      <c r="F87" s="2" t="inlineStr">
         <is>
           <t>Hrdina kopiruje pohyb palca.</t>
         </is>
       </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H86" t="inlineStr">
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
         <is>
           <t>switch|POHYB KOPIRUJE PALEC</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G86"/>
-  <conditionalFormatting sqref="G2:G86">
+  <autoFilter ref="A1:G87"/>
+  <conditionalFormatting sqref="G2:G87">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"A"</formula>
     </cfRule>
@@ -4076,7 +4114,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G86" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"A,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Package 1 step B: floating damage numbers and critical hit (A5 A6); axe-hit buzz 200 ms; note T49 (vibration by attacker)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PANEL_prvky.xlsx
+++ b/PANEL_prvky.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Panel'!$A$1:$G$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Panel'!$A$1:$G$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:H91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1950,7 +1950,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>200.0</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2025,17 +2025,17 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>HUDBA</t>
+          <t>CISLA POSKODENIA</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Zapne/vypne hudbu.</t>
+          <t>Nad zasiahnutym nepriatelom vyleti cislo poskodenia.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>switch|HUDBA</t>
+          <t>switch|CISLA POSKODENIA</t>
         </is>
       </c>
     </row>
@@ -2067,27 +2067,27 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>hlasitost hudby (dB)</t>
+          <t>velkost cisel poskodenia</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>26.0</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Hlasitost hudby.</t>
+          <t>Velkost pisma cisel poskodenia.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>slider|hlasitost hudby (dB)</t>
+          <t>slider|velkost cisel poskodenia</t>
         </is>
       </c>
     </row>
@@ -2109,17 +2109,17 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>ZMRAZIT SVET (hybe sa len hrdina)</t>
+          <t>KRITICKY ZASAH</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Zastavi nepriatelov, kotly a ich strely; hybe sa len hrdina.</t>
+          <t>Cast zasahov je kritickych (2 zivoty, zlte cislo, silnejsie efekty).</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>switch|ZMRAZIT SVET (hybe sa len hrdina)</t>
+          <t>switch|KRITICKY ZASAH</t>
         </is>
       </c>
     </row>
@@ -2146,22 +2146,22 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT BEZCOV</t>
+          <t>sanca na kriticky zasah (%)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat bezci.</t>
+          <t>Kolko percent zasahov je kritickych (100 = vzdy na test).</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>switch|VYPNUT BEZCOV</t>
+          <t>slider|sanca na kriticky zasah (%)</t>
         </is>
       </c>
     </row>
@@ -2193,7 +2193,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT STRELCOV</t>
+          <t>HUDBA</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2203,7 +2203,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat strelci.</t>
+          <t>Zapne/vypne hudbu.</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>switch|VYPNUT STRELCOV</t>
+          <t>switch|HUDBA</t>
         </is>
       </c>
     </row>
@@ -2230,32 +2230,32 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT TUCNAKOV</t>
+          <t>hlasitost hudby (dB)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat tucniaci.</t>
+          <t>Hlasitost hudby.</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>switch|VYPNUT TUCNAKOV</t>
+          <t>slider|hlasitost hudby (dB)</t>
         </is>
       </c>
     </row>
@@ -2272,22 +2272,22 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>kolko bezcov naraz (test)</t>
+          <t>ZMRAZIT SVET (hybe sa len hrdina)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Kolko bezcov je naraz v hre.</t>
+          <t>Zastavi nepriatelov, kotly a ich strely; hybe sa len hrdina.</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>slider|kolko bezcov naraz (test)</t>
+          <t>switch|ZMRAZIT SVET (hybe sa len hrdina)</t>
         </is>
       </c>
     </row>
@@ -2314,22 +2314,22 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>kolko strelcov naraz (test)</t>
+          <t>VYPNUT BEZCOV</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Kolko strelcov je naraz v hre.</t>
+          <t>Nebudu sa objavovat bezci.</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>slider|kolko strelcov naraz (test)</t>
+          <t>switch|VYPNUT BEZCOV</t>
         </is>
       </c>
     </row>
@@ -2356,22 +2356,22 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>kolko tucnakov naraz (test)</t>
+          <t>VYPNUT STRELCOV</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Kolko tucniakov je naraz v hre.</t>
+          <t>Nebudu sa objavovat strelci.</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>slider|kolko tucnakov naraz (test)</t>
+          <t>switch|VYPNUT STRELCOV</t>
         </is>
       </c>
     </row>
@@ -2393,27 +2393,27 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>POHYB</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>posun palca pre plnu rychlost vlavo</t>
+          <t>VYPNUT TUCNAKOV</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Ako daleko od stredu paky treba posunut palec pre plnu rychlost (mensie cislo = rychlejsie plna rychlost, kratsia pomala zona).</t>
+          <t>Nebudu sa objavovat tucniaci.</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>slider|posun palca pre plnu rychlost vlavo</t>
+          <t>switch|VYPNUT TUCNAKOV</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2435,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>POHYB</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2445,17 +2445,17 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>posun palca pre plnu rychlost vpravo</t>
+          <t>kolko bezcov naraz (test)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>15.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>To iste, vpravo; plati aj pre pohyb hore a dole.</t>
+          <t>Kolko bezcov je naraz v hre.</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>slider|posun palca pre plnu rychlost vpravo</t>
+          <t>slider|kolko bezcov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -2477,7 +2477,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>POHYB</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2487,17 +2487,17 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>o kolko pomalsi je pohyb hore-dole</t>
+          <t>kolko strelcov naraz (test)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>1 = hore/dole rovnako rychlo ako do stran; menej = pomalsie.</t>
+          <t>Kolko strelcov je naraz v hre.</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2507,7 +2507,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>slider|o kolko pomalsi je pohyb hore-dole</t>
+          <t>slider|kolko strelcov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -2519,7 +2519,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2529,27 +2529,27 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>ako blizko k postave prestane mierit</t>
+          <t>kolko tucnakov naraz (test)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Mierenie sa vypne, ked je palec blizko postavy.</t>
+          <t>Kolko tucniakov je naraz v hre.</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>slider|ako blizko k postave prestane mierit</t>
+          <t>slider|kolko tucnakov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>POHYB</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2571,17 +2571,17 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>rychlost postavy</t>
+          <t>posun palca pre plnu rychlost vlavo</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti hrdinu.</t>
+          <t>Ako daleko od stredu paky treba posunut palec pre plnu rychlost (mensie cislo = rychlejsie plna rychlost, kratsia pomala zona).</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2591,7 +2591,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>slider|rychlost postavy</t>
+          <t>slider|posun palca pre plnu rychlost vlavo</t>
         </is>
       </c>
     </row>
@@ -2603,7 +2603,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>POHYB</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2613,27 +2613,27 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>pohyb pocas hodu (0 = stoji)</t>
+          <t>posun palca pre plnu rychlost vpravo</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Ako rychlo sa hrdina hybe pocas hodu.</t>
+          <t>To iste, vpravo; plati aj pre pohyb hore a dole.</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>slider|pohyb pocas hodu (0 = stoji)</t>
+          <t>slider|posun palca pre plnu rychlost vpravo</t>
         </is>
       </c>
     </row>
@@ -2645,7 +2645,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>POHYB</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2655,27 +2655,27 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>rychlost zamachu pri hode (1 = povodna)</t>
+          <t>o kolko pomalsi je pohyb hore-dole</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Rychlost animacie hodu.</t>
+          <t>1 = hore/dole rovnako rychlo ako do stran; menej = pomalsie.</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>slider|rychlost zamachu pri hode (1 = povodna)</t>
+          <t>slider|o kolko pomalsi je pohyb hore-dole</t>
         </is>
       </c>
     </row>
@@ -2692,22 +2692,22 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>HRDINA 2x (vypnute = 1x)</t>
+          <t>ako blizko k postave prestane mierit</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Velkost hrdinu.</t>
+          <t>Mierenie sa vypne, ked je palec blizko postavy.</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>switch|HRDINA 2x (vypnute = 1x)</t>
+          <t>slider|ako blizko k postave prestane mierit</t>
         </is>
       </c>
     </row>
@@ -2734,22 +2734,22 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>SEKERA (vypnute = gulky)</t>
+          <t>rychlost postavy</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Prepina zbran: sekera alebo gulky.</t>
+          <t>Nasobok rychlosti hrdinu.</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>switch|SEKERA (vypnute = gulky)</t>
+          <t>slider|rychlost postavy</t>
         </is>
       </c>
     </row>
@@ -2781,27 +2781,27 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>dosah sekery</t>
+          <t>pohyb pocas hodu (0 = stoji)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>350.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Ako daleko sekera doletí.</t>
+          <t>Ako rychlo sa hrdina hybe pocas hodu.</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>slider|dosah sekery</t>
+          <t>slider|pohyb pocas hodu (0 = stoji)</t>
         </is>
       </c>
     </row>
@@ -2823,27 +2823,27 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>rychlost sekery</t>
+          <t>rychlost zamachu pri hode (1 = povodna)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>650.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Rychlost sekery smerom k cielu (spat je 1,5x).</t>
+          <t>Rychlost animacie hodu.</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>slider|rychlost sekery</t>
+          <t>slider|rychlost zamachu pri hode (1 = povodna)</t>
         </is>
       </c>
     </row>
@@ -2860,28 +2860,32 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>NOVE SUDY (postavi ich pred hrdinu)</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr"/>
+          <t>HRDINA 2x (vypnute = 1x)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>ZAP</t>
+        </is>
+      </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Tlacidlo: znova postavi sudy.</t>
+          <t>Velkost hrdinu.</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>button|NOVE SUDY (postavi ich pred hrdinu)</t>
+          <t>switch|HRDINA 2x (vypnute = 1x)</t>
         </is>
       </c>
     </row>
@@ -2898,32 +2902,32 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>aky vysoky kus tela hraca sa da trafit (0-1)</t>
+          <t>SEKERA (vypnute = gulky)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Vyska zasiahnutelnej casti hrdinu.</t>
+          <t>Prepina zbran: sekera alebo gulky.</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>slider|aky vysoky kus tela hraca sa da trafit (0-1)</t>
+          <t>switch|SEKERA (vypnute = gulky)</t>
         </is>
       </c>
     </row>
@@ -2935,7 +2939,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2945,17 +2949,17 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>rychlost bezcov</t>
+          <t>dosah sekery</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>350.0</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti bezcov.</t>
+          <t>Ako daleko sekera doletí.</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2965,7 +2969,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>slider|rychlost bezcov</t>
+          <t>slider|dosah sekery</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2981,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2987,17 +2991,17 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>rychlost strelcov</t>
+          <t>rychlost sekery</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>650.0</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti strelcov.</t>
+          <t>Rychlost sekery smerom k cielu (spat je 1,5x).</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3007,7 +3011,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>slider|rychlost strelcov</t>
+          <t>slider|rychlost sekery</t>
         </is>
       </c>
     </row>
@@ -3019,37 +3023,33 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>button</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>na aku vzdialenost si bezec vsimne hraca (px)</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>640.0</t>
-        </is>
-      </c>
+          <t>NOVE SUDY (postavi ich pred hrdinu)</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Dosah, od ktoreho bezec zacne prenasledovat.</t>
+          <t>Tlacidlo: znova postavi sudy.</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>slider|na aku vzdialenost si bezec vsimne hraca (px)</t>
+          <t>button|NOVE SUDY (postavi ich pred hrdinu)</t>
         </is>
       </c>
     </row>
@@ -3061,37 +3061,37 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
+          <t>aky vysoky kus tela hraca sa da trafit (0-1)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Nakresli kruh sekery a obdlzniky zasahu nepriatelov a hrdinu.</t>
+          <t>Vyska zasiahnutelnej casti hrdinu.</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>switch|UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
+          <t>slider|aky vysoky kus tela hraca sa da trafit (0-1)</t>
         </is>
       </c>
     </row>
@@ -3113,17 +3113,17 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>sekera: polomer zasahu (px)</t>
+          <t>rychlost bezcov</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Velkost kruhu sekery; sekera zasiahne kazdeho, koho obdlznik sa dotkne kruhu.</t>
+          <t>Nasobok rychlosti bezcov.</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>slider|sekera: polomer zasahu (px)</t>
+          <t>slider|rychlost bezcov</t>
         </is>
       </c>
     </row>
@@ -3150,32 +3150,32 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>UKAZ ZONU UDERU BEZCA</t>
+          <t>rychlost strelcov</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Nakresli kruh, kam dopadne uder bezca.</t>
+          <t>Nasobok rychlosti strelcov.</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>switch|UKAZ ZONU UDERU BEZCA</t>
+          <t>slider|rychlost strelcov</t>
         </is>
       </c>
     </row>
@@ -3197,17 +3197,17 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
+          <t>na aku vzdialenost si bezec vsimne hraca (px)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>640.0</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Poloha zony uderu.</t>
+          <t>Dosah, od ktoreho bezec zacne prenasledovat.</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3217,7 +3217,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>slider|zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
+          <t>slider|na aku vzdialenost si bezec vsimne hraca (px)</t>
         </is>
       </c>
     </row>
@@ -3234,32 +3234,32 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: vyska dopadu nad nohami bezca (px)</t>
+          <t>UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Poloha zony uderu.</t>
+          <t>Nakresli kruh sekery a obdlzniky zasahu nepriatelov a hrdinu.</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>slider|zona uderu: vyska dopadu nad nohami bezca (px)</t>
+          <t>switch|UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
         </is>
       </c>
     </row>
@@ -3281,27 +3281,27 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
+          <t>sekera: polomer zasahu (px)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Velkost zony uderu.</t>
+          <t>Velkost kruhu sekery; sekera zasiahne kazdeho, koho obdlznik sa dotkne kruhu.</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>slider|zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
+          <t>slider|sekera: polomer zasahu (px)</t>
         </is>
       </c>
     </row>
@@ -3318,22 +3318,22 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
+          <t>UKAZ ZONU UDERU BEZCA</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Casovanie zasahu v animacii.</t>
+          <t>Nakresli kruh, kam dopadne uder bezca.</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3343,7 +3343,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>slider|kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
+          <t>switch|UKAZ ZONU UDERU BEZCA</t>
         </is>
       </c>
     </row>
@@ -3365,17 +3365,17 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
+          <t>zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Vyska zasiahnutelnej casti nepriatela.</t>
+          <t>Poloha zony uderu.</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -3385,7 +3385,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>slider|aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
+          <t>slider|zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
         </is>
       </c>
     </row>
@@ -3402,32 +3402,32 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>PEVNE TELA (nikto cez nikoho neprejde)</t>
+          <t>zona uderu: vyska dopadu nad nohami bezca (px)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Zapne pevne nohy postav; nikto cez nikoho neprejde.</t>
+          <t>Poloha zony uderu.</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>switch|PEVNE TELA (nikto cez nikoho neprejde)</t>
+          <t>slider|zona uderu: vyska dopadu nad nohami bezca (px)</t>
         </is>
       </c>
     </row>
@@ -3449,17 +3449,17 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>pevne telo: hlbka nohy (px; 54 = cele telo)</t>
+          <t>zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Hlbka pevneho tela (odladene 30).</t>
+          <t>Velkost zony uderu.</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3469,7 +3469,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>slider|pevne telo: hlbka nohy (px; 54 = cele telo)</t>
+          <t>slider|zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
         </is>
       </c>
     </row>
@@ -3491,17 +3491,17 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>pevne telo: sirka nohy (px)</t>
+          <t>kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Sirka pevneho tela (odladene 60).</t>
+          <t>Casovanie zasahu v animacii.</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3511,7 +3511,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>slider|pevne telo: sirka nohy (px)</t>
+          <t>slider|kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
         </is>
       </c>
     </row>
@@ -3533,17 +3533,17 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
+          <t>aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Stary mak odtlacania; funguje len ked su PEVNE TELA vypnute.</t>
+          <t>Vyska zasiahnutelnej casti nepriatela.</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3553,7 +3553,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>slider|ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
+          <t>slider|aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
         </is>
       </c>
     </row>
@@ -3565,27 +3565,27 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>bezec odhodi hrdinu (px)</t>
+          <t>PEVNE TELA (nikto cez nikoho neprejde)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu po zasahu bezca.</t>
+          <t>Zapne pevne nohy postav; nikto cez nikoho neprejde.</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3595,7 +3595,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>slider|bezec odhodi hrdinu (px)</t>
+          <t>switch|PEVNE TELA (nikto cez nikoho neprejde)</t>
         </is>
       </c>
     </row>
@@ -3607,7 +3607,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3617,27 +3617,27 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>strela strelca odhodi hrdinu (px)</t>
+          <t>pevne telo: hlbka nohy (px; 54 = cele telo)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu po zasahu strely.</t>
+          <t>Hlbka pevneho tela (odladene 30).</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>slider|strela strelca odhodi hrdinu (px)</t>
+          <t>slider|pevne telo: hlbka nohy (px; 54 = cele telo)</t>
         </is>
       </c>
     </row>
@@ -3649,7 +3649,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3659,27 +3659,27 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>sekera odhodi nepriatela (px)</t>
+          <t>pevne telo: sirka nohy (px)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia nepriatela po zasahu sekery.</t>
+          <t>Sirka pevneho tela (odladene 60).</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>slider|sekera odhodi nepriatela (px)</t>
+          <t>slider|pevne telo: sirka nohy (px)</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3701,27 +3701,27 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>vybuch kotla odhodi hrdinu (px)</t>
+          <t>ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>140.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu pri vybuchu kotla.</t>
+          <t>Stary mak odtlacania; funguje len ked su PEVNE TELA vypnute.</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>slider|vybuch kotla odhodi hrdinu (px)</t>
+          <t>slider|ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
         </is>
       </c>
     </row>
@@ -3743,27 +3743,27 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>odhodenie: ako dlho trva (s)</t>
+          <t>bezec odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>90.0</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Trvanie odhodenia (odladene 0,4).</t>
+          <t>Dlzka odhodenia hrdinu po zasahu bezca.</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>slider|odhodenie: ako dlho trva (s)</t>
+          <t>slider|bezec odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -3775,7 +3775,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>ODHODENIE PO ZASAHU</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3785,17 +3785,17 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+          <t>strela strelca odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Zivoty nad postavami.</t>
+          <t>Dlzka odhodenia hrdinu po zasahu strely.</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3805,7 +3805,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>slider|srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+          <t>slider|strela strelca odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -3817,7 +3817,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>ODHODENIE PO ZASAHU</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3827,27 +3827,27 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>tien pod postavami: sila (0 = vypnuty)</t>
+          <t>sekera odhodi nepriatela (px)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Sila tiena (odladene 0,3).</t>
+          <t>Dlzka odhodenia nepriatela po zasahu sekery.</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>slider|tien pod postavami: sila (0 = vypnuty)</t>
+          <t>slider|sekera odhodi nepriatela (px)</t>
         </is>
       </c>
     </row>
@@ -3859,7 +3859,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>ODHODENIE PO ZASAHU</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3869,27 +3869,27 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>tien pod postavami: velkost (x)</t>
+          <t>vybuch kotla odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>140.0</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Velkost tiena (odladene 1).</t>
+          <t>Dlzka odhodenia hrdinu pri vybuchu kotla.</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>slider|tien pod postavami: velkost (x)</t>
+          <t>slider|vybuch kotla odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -3901,7 +3901,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>ODHODENIE PO ZASAHU</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3911,17 +3911,17 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>sirka</t>
+          <t>odhodenie: ako dlho trva (s)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Sirka zony pre lavy palec.</t>
+          <t>Trvanie odhodenia (odladene 0,4).</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>slider|sirka</t>
+          <t>slider|odhodenie: ako dlho trva (s)</t>
         </is>
       </c>
     </row>
@@ -3943,7 +3943,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>SRDIECKA A TIENE</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -3953,27 +3953,27 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>kolko zospodu patri miereniu</t>
+          <t>srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Spodna cast zony patri miereniu.</t>
+          <t>Zivoty nad postavami.</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>slider|kolko zospodu patri miereniu</t>
+          <t>slider|srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
         </is>
       </c>
     </row>
@@ -3985,27 +3985,27 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>SRDIECKA A TIENE</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>MIERIT OD POSTAVY</t>
+          <t>tien pod postavami: sila (0 = vypnuty)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Mierenie zacina od postavy.</t>
+          <t>Sila tiena (odladene 0,3).</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -4015,7 +4015,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>switch|MIERIT OD POSTAVY</t>
+          <t>slider|tien pod postavami: sila (0 = vypnuty)</t>
         </is>
       </c>
     </row>
@@ -4027,27 +4027,27 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>SRDIECKA A TIENE</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>VOLNY POHYB (bez skoku)</t>
+          <t>tien pod postavami: velkost (x)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Hrdina nechodi skokom k prstu.</t>
+          <t>Velkost tiena (odladene 1).</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -4057,7 +4057,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>switch|VOLNY POHYB (bez skoku)</t>
+          <t>slider|tien pod postavami: velkost (x)</t>
         </is>
       </c>
     </row>
@@ -4074,38 +4074,206 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>sirka</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>Sirka zony pre lavy palec.</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>slider|sirka</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>S87</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>kolko zospodu patri miereniu</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>0.16</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Spodna cast zony patri miereniu.</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>slider|kolko zospodu patri miereniu</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>S88</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
           <t>switch</t>
         </is>
       </c>
-      <c r="D87" s="2" t="inlineStr">
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>MIERIT OD POSTAVY</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>ZAP</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>Mierenie zacina od postavy.</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>switch|MIERIT OD POSTAVY</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>S89</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>switch</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>VOLNY POHYB (bez skoku)</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>ZAP</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>Hrdina nechodi skokom k prstu.</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>switch|VOLNY POHYB (bez skoku)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>S90</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>switch</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
         <is>
           <t>POHYB KOPIRUJE PALEC</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
+      <c r="E91" t="inlineStr">
         <is>
           <t>VYP</t>
         </is>
       </c>
-      <c r="F87" s="2" t="inlineStr">
+      <c r="F91" s="2" t="inlineStr">
         <is>
           <t>Hrdina kopiruje pohyb palca.</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H87" t="inlineStr">
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
         <is>
           <t>switch|POHYB KOPIRUJE PALEC</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G87"/>
-  <conditionalFormatting sqref="G2:G87">
+  <autoFilter ref="A1:G91"/>
+  <conditionalFormatting sqref="G2:G91">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"A"</formula>
     </cfRule>
@@ -4114,7 +4282,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G87" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"A,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Close package 1 (Uder ma vahu): archive A1-A6 A8 E1 P1 A14, package 2 is next; default game without brutes and with 1 gunman
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PANEL_prvky.xlsx
+++ b/PANEL_prvky.xlsx
@@ -2408,7 +2408,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -2492,7 +2492,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Package 3: enemy dirt variants (5 baked per kind, panel switch + slider), preview tool, panel catalog refresh
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014j5P4SqpYW49SirSP3JAGF
</commit_message>
<xml_diff>
--- a/PANEL_prvky.xlsx
+++ b/PANEL_prvky.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Panel'!$A$1:$G$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Panel'!$A$1:$G$106</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>12.0</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1063,27 +1063,27 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>kotol: odpocet do vybuchu (s)</t>
+          <t>ako dlho lezia trosky (s)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Za kolko sekund kotol vybuchne po zasahu.</t>
+          <t>Ako dlho ostanú na zemi trosky sudov, hrncov a kotlov, kým zmiznú (náhodne ±25 %).</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>slider|kotol: odpocet do vybuchu (s)</t>
+          <t>slider|ako dlho lezia trosky (s)</t>
         </is>
       </c>
     </row>
@@ -1105,17 +1105,17 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>kotol: dosah vybuchu</t>
+          <t>kotol: odpocet do vybuchu (s)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>220.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Polomer vybuchu kotla v px.</t>
+          <t>Za kolko sekund kotol vybuchne po zasahu.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>slider|kotol: dosah vybuchu</t>
+          <t>slider|kotol: odpocet do vybuchu (s)</t>
         </is>
       </c>
     </row>
@@ -1142,22 +1142,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>VYBUCH ZRANI AJ HRDINU</t>
+          <t>kotol: dosah vybuchu</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>220.0</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Ak je vypnute, vybuch kotla zraňuje len nepriatelov.</t>
+          <t>Polomer vybuchu kotla v px.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>switch|VYBUCH ZRANI AJ HRDINU</t>
+          <t>slider|kotol: dosah vybuchu</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>ZVUKY</t>
+          <t>VYBUCH ZRANI AJ HRDINU</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Zapne/vypne zvukove efekty.</t>
+          <t>Ak je vypnute, vybuch kotla zraňuje len nepriatelov.</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>switch|ZVUKY</t>
+          <t>switch|VYBUCH ZRANI AJ HRDINU</t>
         </is>
       </c>
     </row>
@@ -1226,32 +1226,32 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>hlasitost efektov (dB)</t>
+          <t>ZVUKY</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Hlasitost zvukovych efektov.</t>
+          <t>Zapne/vypne zvukove efekty.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>slider|hlasitost efektov (dB)</t>
+          <t>switch|ZVUKY</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1273,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>hlasitost hlasov (dB)</t>
+          <t>hlasitost efektov (dB)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Hlasitost hlasov nepriatelov.</t>
+          <t>Hlasitost zvukovych efektov.</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1293,7 +1293,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>slider|hlasitost hlasov (dB)</t>
+          <t>slider|hlasitost efektov (dB)</t>
         </is>
       </c>
     </row>
@@ -1315,17 +1315,17 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>nahodnost efektov: hlasitost +- (dB)</t>
+          <t>hlasitost hlasov (dB)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Nahodna zmena hlasitosti (odladene 2,5).</t>
+          <t>Hlasitost hlasov nepriatelov.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1335,7 +1335,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>slider|nahodnost efektov: hlasitost +- (dB)</t>
+          <t>slider|hlasitost hlasov (dB)</t>
         </is>
       </c>
     </row>
@@ -1357,17 +1357,17 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>nahodnost efektov: vyska tonu +- (%)</t>
+          <t>nahodnost efektov: hlasitost +- (dB)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>25.0</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Nahodna zmena vysky tonu (odladene 25).</t>
+          <t>Nahodna zmena hlasitosti (odladene 2,5).</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>slider|nahodnost efektov: vyska tonu +- (%)</t>
+          <t>slider|nahodnost efektov: hlasitost +- (dB)</t>
         </is>
       </c>
     </row>
@@ -1399,17 +1399,17 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>ako casto hovoria nepriatelia (s)</t>
+          <t>nahodnost efektov: vyska tonu +- (%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>25.0</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Interval hlasok nepriatelov.</t>
+          <t>Nahodna zmena vysky tonu (odladene 25).</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>slider|ako casto hovoria nepriatelia (s)</t>
+          <t>slider|nahodnost efektov: vyska tonu +- (%)</t>
         </is>
       </c>
     </row>
@@ -1436,22 +1436,22 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>VIBRACIE</t>
+          <t>ako casto hovoria nepriatelia (s)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Vibracie telefonu pri zasahu.</t>
+          <t>Interval hlasok nepriatelov.</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1461,7 +1461,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>switch|VIBRACIE</t>
+          <t>slider|ako casto hovoria nepriatelia (s)</t>
         </is>
       </c>
     </row>
@@ -1478,22 +1478,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>sila vibracii</t>
+          <t>VIBRACIE</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Sila vibracie.</t>
+          <t>Vibracie telefonu pri zasahu.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>slider|sila vibracii</t>
+          <t>switch|VIBRACIE</t>
         </is>
       </c>
     </row>
@@ -1525,17 +1525,17 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>dlzka vibracie pri zasahu (ms)</t>
+          <t>sila vibracii</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>180.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Dlzka vibracie.</t>
+          <t>Sila vibracie.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>slider|dlzka vibracie pri zasahu (ms)</t>
+          <t>slider|sila vibracii</t>
         </is>
       </c>
     </row>
@@ -1562,32 +1562,32 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>ZASTAVENIE PRI ZASAHU</t>
+          <t>dlzka vibracie pri zasahu (ms)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>180.0</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Pri zasahu tvojej zbrane sa hra na okamih zastavi (pocit tazkeho uderu).</t>
+          <t>Dlzka vibracie.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>switch|ZASTAVENIE PRI ZASAHU</t>
+          <t>slider|dlzka vibracie pri zasahu (ms)</t>
         </is>
       </c>
     </row>
@@ -1604,22 +1604,22 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>zastavenie pri zasahu (ms)</t>
+          <t>ZASTAVENIE PRI ZASAHU</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Ako dlho trva zastavenie pri zasahu (pri zabiti dlhsie).</t>
+          <t>Pri zasahu tvojej zbrane sa hra na okamih zastavi (pocit tazkeho uderu).</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>slider|zastavenie pri zasahu (ms)</t>
+          <t>switch|ZASTAVENIE PRI ZASAHU</t>
         </is>
       </c>
     </row>
@@ -1646,22 +1646,22 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>BIELY ZABLESK</t>
+          <t>zastavenie pri zasahu (ms)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Zasiahnuty nepriatel na chvilu cely zbeli.</t>
+          <t>Ako dlho trva zastavenie pri zasahu (pri zabiti dlhsie).</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>switch|BIELY ZABLESK</t>
+          <t>slider|zastavenie pri zasahu (ms)</t>
         </is>
       </c>
     </row>
@@ -1688,22 +1688,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>dlzka bieleho zablesku (ms)</t>
+          <t>BIELY ZABLESK</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Ako dlho je nepriatel biely.</t>
+          <t>Zasiahnuty nepriatel na chvilu cely zbeli.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1713,7 +1713,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>slider|dlzka bieleho zablesku (ms)</t>
+          <t>switch|BIELY ZABLESK</t>
         </is>
       </c>
     </row>
@@ -1730,22 +1730,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>TRASENIE OBRAZU PRI ZASAHU</t>
+          <t>dlzka bieleho zablesku (ms)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Obrazovka sa zatrasie pri zasahu a zabiti sekerou.</t>
+          <t>Ako dlho je nepriatel biely.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>switch|TRASENIE OBRAZU PRI ZASAHU</t>
+          <t>slider|dlzka bieleho zablesku (ms)</t>
         </is>
       </c>
     </row>
@@ -1772,22 +1772,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>sila trasenia pri zasahu</t>
+          <t>TRASENIE OBRAZU PRI ZASAHU</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Nasobok sily trasenia (1.0 = zakladna).</t>
+          <t>Obrazovka sa zatrasie pri zasahu a zabiti sekerou.</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>slider|sila trasenia pri zasahu</t>
+          <t>switch|TRASENIE OBRAZU PRI ZASAHU</t>
         </is>
       </c>
     </row>
@@ -1814,22 +1814,22 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>KOPNUTIE KAMERY</t>
+          <t>sila trasenia pri zasahu</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>Kamera sa na okamih trhne v smere letu seker/strely.</t>
+          <t>Nasobok sily trasenia (1.0 = zakladna).</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>switch|KOPNUTIE KAMERY</t>
+          <t>slider|sila trasenia pri zasahu</t>
         </is>
       </c>
     </row>
@@ -1856,22 +1856,22 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>sila kopnutia kamery</t>
+          <t>KOPNUTIE KAMERY</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Nasobok sily kopnutia (1.0 = zakladna).</t>
+          <t>Kamera sa na okamih trhne v smere letu seker/strely.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1881,7 +1881,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>slider|sila kopnutia kamery</t>
+          <t>switch|KOPNUTIE KAMERY</t>
         </is>
       </c>
     </row>
@@ -1898,22 +1898,22 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>VIBRACIA PRI MOJOM ZASAHU</t>
+          <t>sila kopnutia kamery</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Kratke zavibrovanie telefonu, ked tvoja zbran zasiahne nepriatela.</t>
+          <t>Nasobok sily kopnutia (1.0 = zakladna).</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>switch|VIBRACIA PRI MOJOM ZASAHU</t>
+          <t>slider|sila kopnutia kamery</t>
         </is>
       </c>
     </row>
@@ -1940,22 +1940,22 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>dlzka vibracie pri mojom zasahu (ms)</t>
+          <t>VIBRACIA PRI MOJOM ZASAHU</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>200.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Dlzka vibracie pri tvojom zasahu.</t>
+          <t>Kratke zavibrovanie telefonu, ked tvoja zbran zasiahne nepriatela.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>slider|dlzka vibracie pri mojom zasahu (ms)</t>
+          <t>switch|VIBRACIA PRI MOJOM ZASAHU</t>
         </is>
       </c>
     </row>
@@ -1982,18 +1982,22 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>TEST VIBRACIE (rovnaka ako pri mojom zasahu)</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr"/>
+          <t>dlzka vibracie pri mojom zasahu (ms)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>200.0</t>
+        </is>
+      </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Tlacidlo: jedna vibracia presne taka, ako pri tvojom zasahu (na zistenie, ci telefon vibruje).</t>
+          <t>Dlzka vibracie pri tvojom zasahu.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2003,7 +2007,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>button|TEST VIBRACIE (rovnaka ako pri mojom zasahu)</t>
+          <t>slider|dlzka vibracie pri mojom zasahu (ms)</t>
         </is>
       </c>
     </row>
@@ -2025,7 +2029,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>CISLA POSKODENIA</t>
+          <t>TELO PO SMRTI</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2035,7 +2039,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Nad zasiahnutym nepriatelom vyleti cislo poskodenia.</t>
+          <t>Zabity nepriatel odleti v smere uderu, pretoci sa, dopadne a poskoci; telo chvilu lezi.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2045,7 +2049,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>switch|CISLA POSKODENIA</t>
+          <t>switch|TELO PO SMRTI</t>
         </is>
       </c>
     </row>
@@ -2067,17 +2071,17 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>velkost cisel poskodenia</t>
+          <t>sila odletu tela</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Velkost pisma cisel poskodenia.</t>
+          <t>Nasobok sily odletu tela (1 = zakladna).</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2087,7 +2091,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>slider|velkost cisel poskodenia</t>
+          <t>slider|sila odletu tela</t>
         </is>
       </c>
     </row>
@@ -2104,22 +2108,22 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>KRITICKY ZASAH</t>
+          <t>rychlost animacie padu (fps)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Cast zasahov je kritickych (2 zivoty, zlte cislo, silnejsie efekty).</t>
+          <t>Ako rychlo sa prehra animacia padu bezca (12 = asi pol sekundy).</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2129,7 +2133,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>switch|KRITICKY ZASAH</t>
+          <t>slider|rychlost animacie padu (fps)</t>
         </is>
       </c>
     </row>
@@ -2151,17 +2155,17 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>sanca na kriticky zasah (%)</t>
+          <t>ako dlho telo lezi (s)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>15.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Kolko percent zasahov je kritickych (100 = vzdy na test).</t>
+          <t>Kolko sekund telo lezi, kym zmizne.</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2171,7 +2175,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>slider|sanca na kriticky zasah (%)</t>
+          <t>slider|ako dlho telo lezi (s)</t>
         </is>
       </c>
     </row>
@@ -2193,17 +2197,17 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>HUDBA</t>
+          <t>TELO ZMIZNE V DYME</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Zapne/vypne hudbu.</t>
+          <t>Telo zmizne v oblaku dymu (vypnute = len sa vytrati).</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2213,7 +2217,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>switch|HUDBA</t>
+          <t>switch|TELO ZMIZNE V DYME</t>
         </is>
       </c>
     </row>
@@ -2230,32 +2234,32 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>hlasitost hudby (dB)</t>
+          <t>SPOMALENIE PRI POSLEDNOM ZABITI</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Hlasitost hudby.</t>
+          <t>Cas sa na chvilu spomali po zabiti posledneho nepriatela v boji a po kazdom brutovi.</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>slider|hlasitost hudby (dB)</t>
+          <t>switch|SPOMALENIE PRI POSLEDNOM ZABITI</t>
         </is>
       </c>
     </row>
@@ -2272,22 +2276,22 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>ZMRAZIT SVET (hybe sa len hrdina)</t>
+          <t>dlzka spomalenia (ms)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>600.0</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Zastavi nepriatelov, kotly a ich strely; hybe sa len hrdina.</t>
+          <t>Ako dlho trva spomalenie (skutocne ms).</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2297,7 +2301,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>switch|ZMRAZIT SVET (hybe sa len hrdina)</t>
+          <t>slider|dlzka spomalenia (ms)</t>
         </is>
       </c>
     </row>
@@ -2314,22 +2318,22 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT BEZCOV</t>
+          <t>rychlost pocas spomalenia</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat bezci.</t>
+          <t>Aky rychly je cas pocas spomalenia (1 = normalne).</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2339,7 +2343,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>switch|VYPNUT BEZCOV</t>
+          <t>slider|rychlost pocas spomalenia</t>
         </is>
       </c>
     </row>
@@ -2356,22 +2360,22 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT STRELCOV</t>
+          <t>spomalenie: max. odstup zabiti (s)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat strelci.</t>
+          <t>Najvacsia pauza medzi zabitiami, aby sa seria nerozpadla.</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2381,7 +2385,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>switch|VYPNUT STRELCOV</t>
+          <t>slider|spomalenie: max. odstup zabiti (s)</t>
         </is>
       </c>
     </row>
@@ -2398,22 +2402,22 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT TUCNAKOV</t>
+          <t>spomalenie: kolko zabiti v serii</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat tucniaci.</t>
+          <t>Kolko zabiti za sebou treba pre spomalenie na poslednom.</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2423,7 +2427,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>switch|VYPNUT TUCNAKOV</t>
+          <t>slider|spomalenie: kolko zabiti v serii</t>
         </is>
       </c>
     </row>
@@ -2445,17 +2449,17 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>kolko bezcov naraz (test)</t>
+          <t>spomalenie: dosah 'posledny' (px)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>900.0</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Kolko bezcov je naraz v hre.</t>
+          <t>V akom okruhu okolo hraca nesmie byt dalsi zivy nepriatel.</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2465,7 +2469,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>slider|kolko bezcov naraz (test)</t>
+          <t>slider|spomalenie: dosah 'posledny' (px)</t>
         </is>
       </c>
     </row>
@@ -2487,7 +2491,7 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>kolko strelcov naraz (test)</t>
+          <t>NAHODNOST (nasobok)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2497,7 +2501,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Kolko strelcov je naraz v hre.</t>
+          <t>Nasobok nahodneho rozptylu pri silach, rychlostiach a dlzkach efektov (1 = dohodnuty, 0 = vypnute).</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2507,7 +2511,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>slider|kolko strelcov naraz (test)</t>
+          <t>slider|NAHODNOST (nasobok)</t>
         </is>
       </c>
     </row>
@@ -2524,22 +2528,22 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>kolko tucnakov naraz (test)</t>
+          <t>SPINA NA NEPRIATELOCH</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Kolko tucniakov je naraz v hre.</t>
+          <t>Nepriatelia maju pri zjaveni jeden z 5 vzhladov s malymi blatovymi skvrnami (aj po smrti).</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2549,7 +2553,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>slider|kolko tucnakov naraz (test)</t>
+          <t>switch|SPINA NA NEPRIATELOCH</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2565,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>POHYB</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2571,17 +2575,17 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>posun palca pre plnu rychlost vlavo</t>
+          <t>spina: pocet skvrn na nepriatela</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>32.0</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Ako daleko od stredu paky treba posunut palec pre plnu rychlost (mensie cislo = rychlejsie plna rychlost, kratsia pomala zona).</t>
+          <t>Kolko skvrn ma kazdy nepriatel (0 = ziadne; nasobi to aj NAHODNOST).</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2591,7 +2595,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>slider|posun palca pre plnu rychlost vlavo</t>
+          <t>slider|spina: pocet skvrn na nepriatela</t>
         </is>
       </c>
     </row>
@@ -2603,27 +2607,23 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>POHYB</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>button</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>posun palca pre plnu rychlost vpravo</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>15.0</t>
-        </is>
-      </c>
+          <t>TEST VIBRACIE (rovnaka ako pri mojom zasahu)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>To iste, vpravo; plati aj pre pohyb hore a dole.</t>
+          <t>Tlacidlo: jedna vibracia presne taka, ako pri tvojom zasahu (na zistenie, ci telefon vibruje).</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>slider|posun palca pre plnu rychlost vpravo</t>
+          <t>button|TEST VIBRACIE (rovnaka ako pri mojom zasahu)</t>
         </is>
       </c>
     </row>
@@ -2645,27 +2645,27 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>POHYB</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>o kolko pomalsi je pohyb hore-dole</t>
+          <t>CISLA POSKODENIA</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>1 = hore/dole rovnako rychlo ako do stran; menej = pomalsie.</t>
+          <t>Nad zasiahnutym nepriatelom vyleti cislo poskodenia.</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2675,7 +2675,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>slider|o kolko pomalsi je pohyb hore-dole</t>
+          <t>switch|CISLA POSKODENIA</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2697,27 +2697,27 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>ako blizko k postave prestane mierit</t>
+          <t>velkost cisel poskodenia</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Mierenie sa vypne, ked je palec blizko postavy.</t>
+          <t>Velkost pisma cisel poskodenia.</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>slider|ako blizko k postave prestane mierit</t>
+          <t>slider|velkost cisel poskodenia</t>
         </is>
       </c>
     </row>
@@ -2729,27 +2729,27 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>rychlost postavy</t>
+          <t>KRITICKY ZASAH</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti hrdinu.</t>
+          <t>Cast zasahov je kritickych (2 zivoty, zlte cislo, silnejsie efekty).</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>slider|rychlost postavy</t>
+          <t>switch|KRITICKY ZASAH</t>
         </is>
       </c>
     </row>
@@ -2771,7 +2771,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2781,27 +2781,27 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>pohyb pocas hodu (0 = stoji)</t>
+          <t>sanca na kriticky zasah (%)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Ako rychlo sa hrdina hybe pocas hodu.</t>
+          <t>Kolko percent zasahov je kritickych (100 = vzdy na test).</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>slider|pohyb pocas hodu (0 = stoji)</t>
+          <t>slider|sanca na kriticky zasah (%)</t>
         </is>
       </c>
     </row>
@@ -2813,37 +2813,37 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>rychlost zamachu pri hode (1 = povodna)</t>
+          <t>HUDBA</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Rychlost animacie hodu.</t>
+          <t>Zapne/vypne hudbu.</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>slider|rychlost zamachu pri hode (1 = povodna)</t>
+          <t>switch|HUDBA</t>
         </is>
       </c>
     </row>
@@ -2855,27 +2855,27 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>HRDINA 2x (vypnute = 1x)</t>
+          <t>hlasitost hudby (dB)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Velkost hrdinu.</t>
+          <t>Hlasitost hudby.</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>switch|HRDINA 2x (vypnute = 1x)</t>
+          <t>slider|hlasitost hudby (dB)</t>
         </is>
       </c>
     </row>
@@ -2897,7 +2897,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2907,17 +2907,17 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>SEKERA (vypnute = gulky)</t>
+          <t>ZMRAZIT SVET (hybe sa len hrdina)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Prepina zbran: sekera alebo gulky.</t>
+          <t>Zastavi nepriatelov, kotly a ich strely; hybe sa len hrdina.</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2927,7 +2927,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>switch|SEKERA (vypnute = gulky)</t>
+          <t>switch|ZMRAZIT SVET (hybe sa len hrdina)</t>
         </is>
       </c>
     </row>
@@ -2939,27 +2939,27 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>dosah sekery</t>
+          <t>VYPNUT BEZCOV</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>350.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Ako daleko sekera doletí.</t>
+          <t>Nebudu sa objavovat bezci.</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>slider|dosah sekery</t>
+          <t>switch|VYPNUT BEZCOV</t>
         </is>
       </c>
     </row>
@@ -2981,27 +2981,27 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>rychlost sekery</t>
+          <t>VYPNUT STRELCOV</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>650.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Rychlost sekery smerom k cielu (spat je 1,5x).</t>
+          <t>Nebudu sa objavovat strelci.</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>slider|rychlost sekery</t>
+          <t>switch|VYPNUT STRELCOV</t>
         </is>
       </c>
     </row>
@@ -3023,23 +3023,27 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>NOVE SUDY (postavi ich pred hrdinu)</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr"/>
+          <t>VYPNUT TUCNAKOV</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>ZAP</t>
+        </is>
+      </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Tlacidlo: znova postavi sudy.</t>
+          <t>Nebudu sa objavovat tucniaci.</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3049,7 +3053,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>button|NOVE SUDY (postavi ich pred hrdinu)</t>
+          <t>switch|VYPNUT TUCNAKOV</t>
         </is>
       </c>
     </row>
@@ -3061,7 +3065,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3071,27 +3075,27 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>aky vysoky kus tela hraca sa da trafit (0-1)</t>
+          <t>kolko bezcov naraz (test)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Vyska zasiahnutelnej casti hrdinu.</t>
+          <t>Kolko bezcov je naraz v hre.</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>slider|aky vysoky kus tela hraca sa da trafit (0-1)</t>
+          <t>slider|kolko bezcov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3107,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3113,7 +3117,7 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>rychlost bezcov</t>
+          <t>kolko strelcov naraz (test)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3123,7 +3127,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti bezcov.</t>
+          <t>Kolko strelcov je naraz v hre.</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3133,7 +3137,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>slider|rychlost bezcov</t>
+          <t>slider|kolko strelcov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -3145,7 +3149,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3155,7 +3159,7 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>rychlost strelcov</t>
+          <t>kolko tucnakov naraz (test)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -3165,7 +3169,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti strelcov.</t>
+          <t>Kolko tucniakov je naraz v hre.</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3175,7 +3179,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>slider|rychlost strelcov</t>
+          <t>slider|kolko tucnakov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -3187,7 +3191,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>POHYB</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3197,27 +3201,27 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>na aku vzdialenost si bezec vsimne hraca (px)</t>
+          <t>posun palca pre plnu rychlost vlavo</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>640.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Dosah, od ktoreho bezec zacne prenasledovat.</t>
+          <t>Ako daleko od stredu paky treba posunut palec pre plnu rychlost (mensie cislo = rychlejsie plna rychlost, kratsia pomala zona).</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>slider|na aku vzdialenost si bezec vsimne hraca (px)</t>
+          <t>slider|posun palca pre plnu rychlost vlavo</t>
         </is>
       </c>
     </row>
@@ -3229,27 +3233,27 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>POHYB</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
+          <t>posun palca pre plnu rychlost vpravo</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Nakresli kruh sekery a obdlzniky zasahu nepriatelov a hrdinu.</t>
+          <t>To iste, vpravo; plati aj pre pohyb hore a dole.</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3259,7 +3263,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>switch|UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
+          <t>slider|posun palca pre plnu rychlost vpravo</t>
         </is>
       </c>
     </row>
@@ -3271,7 +3275,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>POHYB</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3281,17 +3285,17 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>sekera: polomer zasahu (px)</t>
+          <t>o kolko pomalsi je pohyb hore-dole</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Velkost kruhu sekery; sekera zasiahne kazdeho, koho obdlznik sa dotkne kruhu.</t>
+          <t>1 = hore/dole rovnako rychlo ako do stran; menej = pomalsie.</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3301,7 +3305,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>slider|sekera: polomer zasahu (px)</t>
+          <t>slider|o kolko pomalsi je pohyb hore-dole</t>
         </is>
       </c>
     </row>
@@ -3313,27 +3317,27 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>UKAZ ZONU UDERU BEZCA</t>
+          <t>ako blizko k postave prestane mierit</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Nakresli kruh, kam dopadne uder bezca.</t>
+          <t>Mierenie sa vypne, ked je palec blizko postavy.</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3343,7 +3347,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>switch|UKAZ ZONU UDERU BEZCA</t>
+          <t>slider|ako blizko k postave prestane mierit</t>
         </is>
       </c>
     </row>
@@ -3355,7 +3359,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3365,27 +3369,27 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
+          <t>rychlost postavy</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Poloha zony uderu.</t>
+          <t>Nasobok rychlosti hrdinu.</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>slider|zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
+          <t>slider|rychlost postavy</t>
         </is>
       </c>
     </row>
@@ -3397,7 +3401,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3407,17 +3411,17 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: vyska dopadu nad nohami bezca (px)</t>
+          <t>pohyb pocas hodu (0 = stoji)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Poloha zony uderu.</t>
+          <t>Ako rychlo sa hrdina hybe pocas hodu.</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3427,7 +3431,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>slider|zona uderu: vyska dopadu nad nohami bezca (px)</t>
+          <t>slider|pohyb pocas hodu (0 = stoji)</t>
         </is>
       </c>
     </row>
@@ -3439,7 +3443,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3449,17 +3453,17 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
+          <t>rychlost zamachu pri hode (1 = povodna)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Velkost zony uderu.</t>
+          <t>Rychlost animacie hodu.</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3469,7 +3473,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>slider|zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
+          <t>slider|rychlost zamachu pri hode (1 = povodna)</t>
         </is>
       </c>
     </row>
@@ -3481,27 +3485,27 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
+          <t>HRDINA 2x (vypnute = 1x)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Casovanie zasahu v animacii.</t>
+          <t>Velkost hrdinu.</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3511,7 +3515,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>slider|kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
+          <t>switch|HRDINA 2x (vypnute = 1x)</t>
         </is>
       </c>
     </row>
@@ -3523,37 +3527,37 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
+          <t>SEKERA (vypnute = gulky)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Vyska zasiahnutelnej casti nepriatela.</t>
+          <t>Prepina zbran: sekera alebo gulky.</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>slider|aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
+          <t>switch|SEKERA (vypnute = gulky)</t>
         </is>
       </c>
     </row>
@@ -3565,27 +3569,27 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>PEVNE TELA (nikto cez nikoho neprejde)</t>
+          <t>dosah sekery</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>350.0</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Zapne pevne nohy postav; nikto cez nikoho neprejde.</t>
+          <t>Ako daleko sekera doletí.</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3595,7 +3599,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>switch|PEVNE TELA (nikto cez nikoho neprejde)</t>
+          <t>slider|dosah sekery</t>
         </is>
       </c>
     </row>
@@ -3607,7 +3611,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3617,27 +3621,27 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>pevne telo: hlbka nohy (px; 54 = cele telo)</t>
+          <t>rychlost sekery</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>650.0</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Hlbka pevneho tela (odladene 30).</t>
+          <t>Rychlost sekery smerom k cielu (spat je 1,5x).</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>slider|pevne telo: hlbka nohy (px; 54 = cele telo)</t>
+          <t>slider|rychlost sekery</t>
         </is>
       </c>
     </row>
@@ -3649,37 +3653,33 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>button</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>pevne telo: sirka nohy (px)</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>60.0</t>
-        </is>
-      </c>
+          <t>NOVE SUDY (postavi ich pred hrdinu)</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr"/>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Sirka pevneho tela (odladene 60).</t>
+          <t>Tlacidlo: znova postavi sudy.</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>slider|pevne telo: sirka nohy (px)</t>
+          <t>button|NOVE SUDY (postavi ich pred hrdinu)</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3691,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3701,17 +3701,17 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
+          <t>aky vysoky kus tela hraca sa da trafit (0-1)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Stary mak odtlacania; funguje len ked su PEVNE TELA vypnute.</t>
+          <t>Vyska zasiahnutelnej casti hrdinu.</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3721,7 +3721,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>slider|ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
+          <t>slider|aky vysoky kus tela hraca sa da trafit (0-1)</t>
         </is>
       </c>
     </row>
@@ -3733,7 +3733,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3743,17 +3743,17 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>bezec odhodi hrdinu (px)</t>
+          <t>rychlost bezcov</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu po zasahu bezca.</t>
+          <t>Nasobok rychlosti bezcov.</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>slider|bezec odhodi hrdinu (px)</t>
+          <t>slider|rychlost bezcov</t>
         </is>
       </c>
     </row>
@@ -3775,7 +3775,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3785,17 +3785,17 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>strela strelca odhodi hrdinu (px)</t>
+          <t>rychlost strelcov</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu po zasahu strely.</t>
+          <t>Nasobok rychlosti strelcov.</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3805,7 +3805,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>slider|strela strelca odhodi hrdinu (px)</t>
+          <t>slider|rychlost strelcov</t>
         </is>
       </c>
     </row>
@@ -3817,7 +3817,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3827,27 +3827,27 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>sekera odhodi nepriatela (px)</t>
+          <t>na aku vzdialenost si bezec vsimne hraca (px)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>640.0</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia nepriatela po zasahu sekery.</t>
+          <t>Dosah, od ktoreho bezec zacne prenasledovat.</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>slider|sekera odhodi nepriatela (px)</t>
+          <t>slider|na aku vzdialenost si bezec vsimne hraca (px)</t>
         </is>
       </c>
     </row>
@@ -3859,27 +3859,27 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>vybuch kotla odhodi hrdinu (px)</t>
+          <t>UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>140.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu pri vybuchu kotla.</t>
+          <t>Nakresli kruh sekery a obdlzniky zasahu nepriatelov a hrdinu.</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -3889,7 +3889,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>slider|vybuch kotla odhodi hrdinu (px)</t>
+          <t>switch|UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
         </is>
       </c>
     </row>
@@ -3901,7 +3901,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3911,27 +3911,27 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>odhodenie: ako dlho trva (s)</t>
+          <t>sekera: polomer zasahu (px)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Trvanie odhodenia (odladene 0,4).</t>
+          <t>Velkost kruhu sekery; sekera zasiahne kazdeho, koho obdlznik sa dotkne kruhu.</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>slider|odhodenie: ako dlho trva (s)</t>
+          <t>slider|sekera: polomer zasahu (px)</t>
         </is>
       </c>
     </row>
@@ -3943,37 +3943,37 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+          <t>UKAZ ZONU UDERU BEZCA</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Zivoty nad postavami.</t>
+          <t>Nakresli kruh, kam dopadne uder bezca.</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>slider|srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+          <t>switch|UKAZ ZONU UDERU BEZCA</t>
         </is>
       </c>
     </row>
@@ -3985,7 +3985,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -3995,17 +3995,17 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>tien pod postavami: sila (0 = vypnuty)</t>
+          <t>zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Sila tiena (odladene 0,3).</t>
+          <t>Poloha zony uderu.</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -4015,7 +4015,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>slider|tien pod postavami: sila (0 = vypnuty)</t>
+          <t>slider|zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
         </is>
       </c>
     </row>
@@ -4027,7 +4027,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4037,17 +4037,17 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>tien pod postavami: velkost (x)</t>
+          <t>zona uderu: vyska dopadu nad nohami bezca (px)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Velkost tiena (odladene 1).</t>
+          <t>Poloha zony uderu.</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -4057,7 +4057,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>slider|tien pod postavami: velkost (x)</t>
+          <t>slider|zona uderu: vyska dopadu nad nohami bezca (px)</t>
         </is>
       </c>
     </row>
@@ -4069,7 +4069,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4079,17 +4079,17 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>sirka</t>
+          <t>zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Sirka zony pre lavy palec.</t>
+          <t>Velkost zony uderu.</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -4099,7 +4099,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>slider|sirka</t>
+          <t>slider|zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
         </is>
       </c>
     </row>
@@ -4111,7 +4111,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -4121,17 +4121,17 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>kolko zospodu patri miereniu</t>
+          <t>kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Spodna cast zony patri miereniu.</t>
+          <t>Casovanie zasahu v animacii.</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -4141,7 +4141,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>slider|kolko zospodu patri miereniu</t>
+          <t>slider|kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
         </is>
       </c>
     </row>
@@ -4153,27 +4153,27 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>MIERIT OD POSTAVY</t>
+          <t>aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>Mierenie zacina od postavy.</t>
+          <t>Vyska zasiahnutelnej casti nepriatela.</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>switch|MIERIT OD POSTAVY</t>
+          <t>slider|aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
         </is>
       </c>
     </row>
@@ -4195,7 +4195,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -4205,7 +4205,7 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>VOLNY POHYB (bez skoku)</t>
+          <t>PEVNE TELA (nikto cez nikoho neprejde)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4215,17 +4215,17 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>Hrdina nechodi skokom k prstu.</t>
+          <t>Zapne pevne nohy postav; nikto cez nikoho neprejde.</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>switch|VOLNY POHYB (bez skoku)</t>
+          <t>switch|PEVNE TELA (nikto cez nikoho neprejde)</t>
         </is>
       </c>
     </row>
@@ -4237,43 +4237,673 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
+          <t>NEPRIATELIA</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>pevne telo: hlbka nohy (px; 54 = cele telo)</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>30.0</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>Hlbka pevneho tela (odladene 30).</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>slider|pevne telo: hlbka nohy (px; 54 = cele telo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>S91</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>NEPRIATELIA</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>pevne telo: sirka nohy (px)</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>60.0</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>Sirka pevneho tela (odladene 60).</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>slider|pevne telo: sirka nohy (px)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>S92</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>NEPRIATELIA</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>46.0</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>Stary mak odtlacania; funguje len ked su PEVNE TELA vypnute.</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>slider|ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>S93</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>ODHODENIE PO ZASAHU</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>bezec odhodi hrdinu (px)</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>90.0</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>Dlzka odhodenia hrdinu po zasahu bezca.</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>slider|bezec odhodi hrdinu (px)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>S94</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>ODHODENIE PO ZASAHU</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>strela strelca odhodi hrdinu (px)</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>35.0</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>Dlzka odhodenia hrdinu po zasahu strely.</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>slider|strela strelca odhodi hrdinu (px)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>S95</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>ODHODENIE PO ZASAHU</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>sekera odhodi nepriatela (px)</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>70.0</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>Dlzka odhodenia nepriatela po zasahu sekery.</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>slider|sekera odhodi nepriatela (px)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>S96</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>ODHODENIE PO ZASAHU</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>vybuch kotla odhodi hrdinu (px)</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>140.0</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>Dlzka odhodenia hrdinu pri vybuchu kotla.</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>slider|vybuch kotla odhodi hrdinu (px)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>S97</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>ODHODENIE PO ZASAHU</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>odhodenie: ako dlho trva (s)</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>Trvanie odhodenia (odladene 0,4).</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>slider|odhodenie: ako dlho trva (s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>S98</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>SRDIECKA A TIENE</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>Zivoty nad postavami.</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>slider|srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>S99</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>SRDIECKA A TIENE</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>tien pod postavami: sila (0 = vypnuty)</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>Sila tiena (odladene 0,3).</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>slider|tien pod postavami: sila (0 = vypnuty)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>S100</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>SRDIECKA A TIENE</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>tien pod postavami: velkost (x)</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>Velkost tiena (odladene 1).</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>slider|tien pod postavami: velkost (x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>S101</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
           <t>ZONA PRE LAVY PALEC</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>sirka</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>Sirka zony pre lavy palec.</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>slider|sirka</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>S102</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>kolko zospodu patri miereniu</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>0.16</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>Spodna cast zony patri miereniu.</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>slider|kolko zospodu patri miereniu</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>S103</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
         <is>
           <t>switch</t>
         </is>
       </c>
-      <c r="D91" s="2" t="inlineStr">
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>MIERIT OD POSTAVY</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>ZAP</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>Mierenie zacina od postavy.</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>switch|MIERIT OD POSTAVY</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>S104</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>switch</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>VOLNY POHYB (bez skoku)</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>ZAP</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>Hrdina nechodi skokom k prstu.</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>switch|VOLNY POHYB (bez skoku)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>S105</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>switch</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
         <is>
           <t>POHYB KOPIRUJE PALEC</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
+      <c r="E106" t="inlineStr">
         <is>
           <t>VYP</t>
         </is>
       </c>
-      <c r="F91" s="2" t="inlineStr">
+      <c r="F106" s="2" t="inlineStr">
         <is>
           <t>Hrdina kopiruje pohyb palca.</t>
         </is>
       </c>
-      <c r="G91" t="inlineStr">
+      <c r="G106" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr">
+      <c r="H106" t="inlineStr">
         <is>
           <t>switch|POHYB KOPIRUJE PALEC</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G91"/>
-  <conditionalFormatting sqref="G2:G91">
+  <autoFilter ref="A1:G106"/>
+  <conditionalFormatting sqref="G2:G106">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"A"</formula>
     </cfRule>
@@ -4282,7 +4912,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"A,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Package 3: F2 red blink warning before attacks, D4 per-type warning sounds, brute 0.4 s wind-up before the grab, panel switches and sliders
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014j5P4SqpYW49SirSP3JAGF
</commit_message>
<xml_diff>
--- a/PANEL_prvky.xlsx
+++ b/PANEL_prvky.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Panel'!$A$1:$G$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Panel'!$A$1:$G$110</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H106"/>
+  <dimension ref="A1:H110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2580,7 +2580,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>32.0</t>
+          <t>80.0</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2612,18 +2612,22 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>TEST VIBRACIE (rovnaka ako pri mojom zasahu)</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr"/>
+          <t>VAROVANIE PRED UTOKOM (blikanie)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ZAP</t>
+        </is>
+      </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Tlacidlo: jedna vibracia presne taka, ako pri tvojom zasahu (na zistenie, ci telefon vibruje).</t>
+          <t>Nepriatel pred utokom (udrer bezca, vystrel strelca, chytenie obora) blika do cervena.</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2633,7 +2637,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>button|TEST VIBRACIE (rovnaka ako pri mojom zasahu)</t>
+          <t>switch|VAROVANIE PRED UTOKOM (blikanie)</t>
         </is>
       </c>
     </row>
@@ -2655,7 +2659,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>CISLA POSKODENIA</t>
+          <t>ZVUK VAROVANIA</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2665,7 +2669,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Nad zasiahnutym nepriatelom vyleti cislo poskodenia.</t>
+          <t>Kazdy typ nepriatela zahra svoj zvuk na zaciatku utoku (zatial dockovy syntetizovany zvuk).</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2675,7 +2679,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>switch|CISLA POSKODENIA</t>
+          <t>switch|ZVUK VAROVANIA</t>
         </is>
       </c>
     </row>
@@ -2697,17 +2701,17 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>velkost cisel poskodenia</t>
+          <t>varovanie: sila blikania</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Velkost pisma cisel poskodenia.</t>
+          <t>Ako vyrazne nepriatel blika pred utokom (1 = plne).</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2717,7 +2721,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>slider|velkost cisel poskodenia</t>
+          <t>slider|varovanie: sila blikania</t>
         </is>
       </c>
     </row>
@@ -2734,22 +2738,22 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>KRITICKY ZASAH</t>
+          <t>obor: vymah pred chytenim (s)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Cast zasahov je kritickych (2 zivoty, zlte cislo, silnejsie efekty).</t>
+          <t>Obor sa pred chytenim zastavi, zavrci a blika; vtedy mozes uhnut (0 = chyti okamzite).</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2759,7 +2763,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>switch|KRITICKY ZASAH</t>
+          <t>slider|obor: vymah pred chytenim (s)</t>
         </is>
       </c>
     </row>
@@ -2776,22 +2780,18 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>button</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>sanca na kriticky zasah (%)</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>15.0</t>
-        </is>
-      </c>
+          <t>TEST VIBRACIE (rovnaka ako pri mojom zasahu)</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Kolko percent zasahov je kritickych (100 = vzdy na test).</t>
+          <t>Tlacidlo: jedna vibracia presne taka, ako pri tvojom zasahu (na zistenie, ci telefon vibruje).</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>slider|sanca na kriticky zasah (%)</t>
+          <t>button|TEST VIBRACIE (rovnaka ako pri mojom zasahu)</t>
         </is>
       </c>
     </row>
@@ -2823,17 +2823,17 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>HUDBA</t>
+          <t>CISLA POSKODENIA</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Zapne/vypne hudbu.</t>
+          <t>Nad zasiahnutym nepriatelom vyleti cislo poskodenia.</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>switch|HUDBA</t>
+          <t>switch|CISLA POSKODENIA</t>
         </is>
       </c>
     </row>
@@ -2865,27 +2865,27 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>hlasitost hudby (dB)</t>
+          <t>velkost cisel poskodenia</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>16.0</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Hlasitost hudby.</t>
+          <t>Velkost pisma cisel poskodenia.</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>slider|hlasitost hudby (dB)</t>
+          <t>slider|velkost cisel poskodenia</t>
         </is>
       </c>
     </row>
@@ -2907,17 +2907,17 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>ZMRAZIT SVET (hybe sa len hrdina)</t>
+          <t>KRITICKY ZASAH</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Zastavi nepriatelov, kotly a ich strely; hybe sa len hrdina.</t>
+          <t>Cast zasahov je kritickych (2 zivoty, zlte cislo, silnejsie efekty).</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2927,7 +2927,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>switch|ZMRAZIT SVET (hybe sa len hrdina)</t>
+          <t>switch|KRITICKY ZASAH</t>
         </is>
       </c>
     </row>
@@ -2944,22 +2944,22 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT BEZCOV</t>
+          <t>sanca na kriticky zasah (%)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat bezci.</t>
+          <t>Kolko percent zasahov je kritickych (100 = vzdy na test).</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>switch|VYPNUT BEZCOV</t>
+          <t>slider|sanca na kriticky zasah (%)</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT STRELCOV</t>
+          <t>HUDBA</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat strelci.</t>
+          <t>Zapne/vypne hudbu.</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>switch|VYPNUT STRELCOV</t>
+          <t>switch|HUDBA</t>
         </is>
       </c>
     </row>
@@ -3028,32 +3028,32 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT TUCNAKOV</t>
+          <t>hlasitost hudby (dB)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat tucniaci.</t>
+          <t>Hlasitost hudby.</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>switch|VYPNUT TUCNAKOV</t>
+          <t>slider|hlasitost hudby (dB)</t>
         </is>
       </c>
     </row>
@@ -3070,22 +3070,22 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>kolko bezcov naraz (test)</t>
+          <t>ZMRAZIT SVET (hybe sa len hrdina)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Kolko bezcov je naraz v hre.</t>
+          <t>Zastavi nepriatelov, kotly a ich strely; hybe sa len hrdina.</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>slider|kolko bezcov naraz (test)</t>
+          <t>switch|ZMRAZIT SVET (hybe sa len hrdina)</t>
         </is>
       </c>
     </row>
@@ -3112,22 +3112,22 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>kolko strelcov naraz (test)</t>
+          <t>VYPNUT BEZCOV</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Kolko strelcov je naraz v hre.</t>
+          <t>Nebudu sa objavovat bezci.</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3137,7 +3137,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>slider|kolko strelcov naraz (test)</t>
+          <t>switch|VYPNUT BEZCOV</t>
         </is>
       </c>
     </row>
@@ -3154,22 +3154,22 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>kolko tucnakov naraz (test)</t>
+          <t>VYPNUT STRELCOV</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Kolko tucniakov je naraz v hre.</t>
+          <t>Nebudu sa objavovat strelci.</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3179,7 +3179,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>slider|kolko tucnakov naraz (test)</t>
+          <t>switch|VYPNUT STRELCOV</t>
         </is>
       </c>
     </row>
@@ -3191,27 +3191,27 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>POHYB</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>posun palca pre plnu rychlost vlavo</t>
+          <t>VYPNUT TUCNAKOV</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Ako daleko od stredu paky treba posunut palec pre plnu rychlost (mensie cislo = rychlejsie plna rychlost, kratsia pomala zona).</t>
+          <t>Nebudu sa objavovat tucniaci.</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3221,7 +3221,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>slider|posun palca pre plnu rychlost vlavo</t>
+          <t>switch|VYPNUT TUCNAKOV</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>POHYB</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3243,17 +3243,17 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>posun palca pre plnu rychlost vpravo</t>
+          <t>kolko bezcov naraz (test)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>15.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>To iste, vpravo; plati aj pre pohyb hore a dole.</t>
+          <t>Kolko bezcov je naraz v hre.</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>slider|posun palca pre plnu rychlost vpravo</t>
+          <t>slider|kolko bezcov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>POHYB</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3285,7 +3285,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>o kolko pomalsi je pohyb hore-dole</t>
+          <t>kolko strelcov naraz (test)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3295,7 +3295,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>1 = hore/dole rovnako rychlo ako do stran; menej = pomalsie.</t>
+          <t>Kolko strelcov je naraz v hre.</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3305,7 +3305,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>slider|o kolko pomalsi je pohyb hore-dole</t>
+          <t>slider|kolko strelcov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>TEST</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3327,27 +3327,27 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>ako blizko k postave prestane mierit</t>
+          <t>kolko tucnakov naraz (test)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Mierenie sa vypne, ked je palec blizko postavy.</t>
+          <t>Kolko tucniakov je naraz v hre.</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>slider|ako blizko k postave prestane mierit</t>
+          <t>slider|kolko tucnakov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -3359,7 +3359,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>POHYB</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3369,17 +3369,17 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>rychlost postavy</t>
+          <t>posun palca pre plnu rychlost vlavo</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti hrdinu.</t>
+          <t>Ako daleko od stredu paky treba posunut palec pre plnu rychlost (mensie cislo = rychlejsie plna rychlost, kratsia pomala zona).</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -3389,7 +3389,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>slider|rychlost postavy</t>
+          <t>slider|posun palca pre plnu rychlost vlavo</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>POHYB</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3411,27 +3411,27 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>pohyb pocas hodu (0 = stoji)</t>
+          <t>posun palca pre plnu rychlost vpravo</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Ako rychlo sa hrdina hybe pocas hodu.</t>
+          <t>To iste, vpravo; plati aj pre pohyb hore a dole.</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>slider|pohyb pocas hodu (0 = stoji)</t>
+          <t>slider|posun palca pre plnu rychlost vpravo</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>POHYB</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3453,27 +3453,27 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>rychlost zamachu pri hode (1 = povodna)</t>
+          <t>o kolko pomalsi je pohyb hore-dole</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Rychlost animacie hodu.</t>
+          <t>1 = hore/dole rovnako rychlo ako do stran; menej = pomalsie.</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>slider|rychlost zamachu pri hode (1 = povodna)</t>
+          <t>slider|o kolko pomalsi je pohyb hore-dole</t>
         </is>
       </c>
     </row>
@@ -3490,22 +3490,22 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>HRDINA 2x (vypnute = 1x)</t>
+          <t>ako blizko k postave prestane mierit</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Velkost hrdinu.</t>
+          <t>Mierenie sa vypne, ked je palec blizko postavy.</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>switch|HRDINA 2x (vypnute = 1x)</t>
+          <t>slider|ako blizko k postave prestane mierit</t>
         </is>
       </c>
     </row>
@@ -3532,22 +3532,22 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>SEKERA (vypnute = gulky)</t>
+          <t>rychlost postavy</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Prepina zbran: sekera alebo gulky.</t>
+          <t>Nasobok rychlosti hrdinu.</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -3557,7 +3557,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>switch|SEKERA (vypnute = gulky)</t>
+          <t>slider|rychlost postavy</t>
         </is>
       </c>
     </row>
@@ -3579,27 +3579,27 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>dosah sekery</t>
+          <t>pohyb pocas hodu (0 = stoji)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>350.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Ako daleko sekera doletí.</t>
+          <t>Ako rychlo sa hrdina hybe pocas hodu.</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>slider|dosah sekery</t>
+          <t>slider|pohyb pocas hodu (0 = stoji)</t>
         </is>
       </c>
     </row>
@@ -3621,27 +3621,27 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>rychlost sekery</t>
+          <t>rychlost zamachu pri hode (1 = povodna)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>650.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Rychlost sekery smerom k cielu (spat je 1,5x).</t>
+          <t>Rychlost animacie hodu.</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>slider|rychlost sekery</t>
+          <t>slider|rychlost zamachu pri hode (1 = povodna)</t>
         </is>
       </c>
     </row>
@@ -3658,28 +3658,32 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>NOVE SUDY (postavi ich pred hrdinu)</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr"/>
+          <t>HRDINA 2x (vypnute = 1x)</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>ZAP</t>
+        </is>
+      </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Tlacidlo: znova postavi sudy.</t>
+          <t>Velkost hrdinu.</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>button|NOVE SUDY (postavi ich pred hrdinu)</t>
+          <t>switch|HRDINA 2x (vypnute = 1x)</t>
         </is>
       </c>
     </row>
@@ -3696,32 +3700,32 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>aky vysoky kus tela hraca sa da trafit (0-1)</t>
+          <t>SEKERA (vypnute = gulky)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Vyska zasiahnutelnej casti hrdinu.</t>
+          <t>Prepina zbran: sekera alebo gulky.</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>slider|aky vysoky kus tela hraca sa da trafit (0-1)</t>
+          <t>switch|SEKERA (vypnute = gulky)</t>
         </is>
       </c>
     </row>
@@ -3733,7 +3737,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3743,17 +3747,17 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>rychlost bezcov</t>
+          <t>dosah sekery</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>350.0</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti bezcov.</t>
+          <t>Ako daleko sekera doletí.</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3763,7 +3767,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>slider|rychlost bezcov</t>
+          <t>slider|dosah sekery</t>
         </is>
       </c>
     </row>
@@ -3775,7 +3779,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3785,17 +3789,17 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>rychlost strelcov</t>
+          <t>rychlost sekery</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>650.0</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti strelcov.</t>
+          <t>Rychlost sekery smerom k cielu (spat je 1,5x).</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3805,7 +3809,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>slider|rychlost strelcov</t>
+          <t>slider|rychlost sekery</t>
         </is>
       </c>
     </row>
@@ -3817,37 +3821,33 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>button</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>na aku vzdialenost si bezec vsimne hraca (px)</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>640.0</t>
-        </is>
-      </c>
+          <t>NOVE SUDY (postavi ich pred hrdinu)</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Dosah, od ktoreho bezec zacne prenasledovat.</t>
+          <t>Tlacidlo: znova postavi sudy.</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>slider|na aku vzdialenost si bezec vsimne hraca (px)</t>
+          <t>button|NOVE SUDY (postavi ich pred hrdinu)</t>
         </is>
       </c>
     </row>
@@ -3859,37 +3859,37 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
+          <t>aky vysoky kus tela hraca sa da trafit (0-1)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Nakresli kruh sekery a obdlzniky zasahu nepriatelov a hrdinu.</t>
+          <t>Vyska zasiahnutelnej casti hrdinu.</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>switch|UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
+          <t>slider|aky vysoky kus tela hraca sa da trafit (0-1)</t>
         </is>
       </c>
     </row>
@@ -3911,17 +3911,17 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>sekera: polomer zasahu (px)</t>
+          <t>rychlost bezcov</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Velkost kruhu sekery; sekera zasiahne kazdeho, koho obdlznik sa dotkne kruhu.</t>
+          <t>Nasobok rychlosti bezcov.</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -3931,7 +3931,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>slider|sekera: polomer zasahu (px)</t>
+          <t>slider|rychlost bezcov</t>
         </is>
       </c>
     </row>
@@ -3948,32 +3948,32 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>UKAZ ZONU UDERU BEZCA</t>
+          <t>rychlost strelcov</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Nakresli kruh, kam dopadne uder bezca.</t>
+          <t>Nasobok rychlosti strelcov.</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>switch|UKAZ ZONU UDERU BEZCA</t>
+          <t>slider|rychlost strelcov</t>
         </is>
       </c>
     </row>
@@ -3995,17 +3995,17 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
+          <t>na aku vzdialenost si bezec vsimne hraca (px)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>640.0</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Poloha zony uderu.</t>
+          <t>Dosah, od ktoreho bezec zacne prenasledovat.</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -4015,7 +4015,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>slider|zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
+          <t>slider|na aku vzdialenost si bezec vsimne hraca (px)</t>
         </is>
       </c>
     </row>
@@ -4032,32 +4032,32 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: vyska dopadu nad nohami bezca (px)</t>
+          <t>UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Poloha zony uderu.</t>
+          <t>Nakresli kruh sekery a obdlzniky zasahu nepriatelov a hrdinu.</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>slider|zona uderu: vyska dopadu nad nohami bezca (px)</t>
+          <t>switch|UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
         </is>
       </c>
     </row>
@@ -4079,27 +4079,27 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
+          <t>sekera: polomer zasahu (px)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Velkost zony uderu.</t>
+          <t>Velkost kruhu sekery; sekera zasiahne kazdeho, koho obdlznik sa dotkne kruhu.</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>slider|zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
+          <t>slider|sekera: polomer zasahu (px)</t>
         </is>
       </c>
     </row>
@@ -4116,22 +4116,22 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
+          <t>UKAZ ZONU UDERU BEZCA</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Casovanie zasahu v animacii.</t>
+          <t>Nakresli kruh, kam dopadne uder bezca.</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -4141,7 +4141,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>slider|kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
+          <t>switch|UKAZ ZONU UDERU BEZCA</t>
         </is>
       </c>
     </row>
@@ -4163,17 +4163,17 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
+          <t>zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>Vyska zasiahnutelnej casti nepriatela.</t>
+          <t>Poloha zony uderu.</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>slider|aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
+          <t>slider|zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
         </is>
       </c>
     </row>
@@ -4200,32 +4200,32 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>PEVNE TELA (nikto cez nikoho neprejde)</t>
+          <t>zona uderu: vyska dopadu nad nohami bezca (px)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>Zapne pevne nohy postav; nikto cez nikoho neprejde.</t>
+          <t>Poloha zony uderu.</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>switch|PEVNE TELA (nikto cez nikoho neprejde)</t>
+          <t>slider|zona uderu: vyska dopadu nad nohami bezca (px)</t>
         </is>
       </c>
     </row>
@@ -4247,17 +4247,17 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>pevne telo: hlbka nohy (px; 54 = cele telo)</t>
+          <t>zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>Hlbka pevneho tela (odladene 30).</t>
+          <t>Velkost zony uderu.</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>slider|pevne telo: hlbka nohy (px; 54 = cele telo)</t>
+          <t>slider|zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
         </is>
       </c>
     </row>
@@ -4289,17 +4289,17 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>pevne telo: sirka nohy (px)</t>
+          <t>kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>Sirka pevneho tela (odladene 60).</t>
+          <t>Casovanie zasahu v animacii.</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -4309,7 +4309,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>slider|pevne telo: sirka nohy (px)</t>
+          <t>slider|kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
         </is>
       </c>
     </row>
@@ -4331,17 +4331,17 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
+          <t>aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>Stary mak odtlacania; funguje len ked su PEVNE TELA vypnute.</t>
+          <t>Vyska zasiahnutelnej casti nepriatela.</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -4351,7 +4351,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>slider|ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
+          <t>slider|aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
         </is>
       </c>
     </row>
@@ -4363,27 +4363,27 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>bezec odhodi hrdinu (px)</t>
+          <t>PEVNE TELA (nikto cez nikoho neprejde)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu po zasahu bezca.</t>
+          <t>Zapne pevne nohy postav; nikto cez nikoho neprejde.</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -4393,7 +4393,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>slider|bezec odhodi hrdinu (px)</t>
+          <t>switch|PEVNE TELA (nikto cez nikoho neprejde)</t>
         </is>
       </c>
     </row>
@@ -4405,7 +4405,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -4415,27 +4415,27 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>strela strelca odhodi hrdinu (px)</t>
+          <t>pevne telo: hlbka nohy (px; 54 = cele telo)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu po zasahu strely.</t>
+          <t>Hlbka pevneho tela (odladene 30).</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>slider|strela strelca odhodi hrdinu (px)</t>
+          <t>slider|pevne telo: hlbka nohy (px; 54 = cele telo)</t>
         </is>
       </c>
     </row>
@@ -4447,7 +4447,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -4457,27 +4457,27 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>sekera odhodi nepriatela (px)</t>
+          <t>pevne telo: sirka nohy (px)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia nepriatela po zasahu sekery.</t>
+          <t>Sirka pevneho tela (odladene 60).</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>slider|sekera odhodi nepriatela (px)</t>
+          <t>slider|pevne telo: sirka nohy (px)</t>
         </is>
       </c>
     </row>
@@ -4489,7 +4489,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -4499,27 +4499,27 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>vybuch kotla odhodi hrdinu (px)</t>
+          <t>ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>140.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu pri vybuchu kotla.</t>
+          <t>Stary mak odtlacania; funguje len ked su PEVNE TELA vypnute.</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>slider|vybuch kotla odhodi hrdinu (px)</t>
+          <t>slider|ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
         </is>
       </c>
     </row>
@@ -4541,27 +4541,27 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>odhodenie: ako dlho trva (s)</t>
+          <t>bezec odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>90.0</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>Trvanie odhodenia (odladene 0,4).</t>
+          <t>Dlzka odhodenia hrdinu po zasahu bezca.</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>slider|odhodenie: ako dlho trva (s)</t>
+          <t>slider|bezec odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -4573,7 +4573,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>ODHODENIE PO ZASAHU</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -4583,17 +4583,17 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+          <t>strela strelca odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>Zivoty nad postavami.</t>
+          <t>Dlzka odhodenia hrdinu po zasahu strely.</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -4603,7 +4603,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>slider|srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+          <t>slider|strela strelca odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -4615,7 +4615,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>ODHODENIE PO ZASAHU</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -4625,27 +4625,27 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>tien pod postavami: sila (0 = vypnuty)</t>
+          <t>sekera odhodi nepriatela (px)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>Sila tiena (odladene 0,3).</t>
+          <t>Dlzka odhodenia nepriatela po zasahu sekery.</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>slider|tien pod postavami: sila (0 = vypnuty)</t>
+          <t>slider|sekera odhodi nepriatela (px)</t>
         </is>
       </c>
     </row>
@@ -4657,7 +4657,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>ODHODENIE PO ZASAHU</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -4667,27 +4667,27 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>tien pod postavami: velkost (x)</t>
+          <t>vybuch kotla odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>140.0</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Velkost tiena (odladene 1).</t>
+          <t>Dlzka odhodenia hrdinu pri vybuchu kotla.</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>slider|tien pod postavami: velkost (x)</t>
+          <t>slider|vybuch kotla odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -4699,7 +4699,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>ODHODENIE PO ZASAHU</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -4709,17 +4709,17 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>sirka</t>
+          <t>odhodenie: ako dlho trva (s)</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>Sirka zony pre lavy palec.</t>
+          <t>Trvanie odhodenia (odladene 0,4).</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -4729,7 +4729,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>slider|sirka</t>
+          <t>slider|odhodenie: ako dlho trva (s)</t>
         </is>
       </c>
     </row>
@@ -4741,7 +4741,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>SRDIECKA A TIENE</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -4751,27 +4751,27 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>kolko zospodu patri miereniu</t>
+          <t>srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>Spodna cast zony patri miereniu.</t>
+          <t>Zivoty nad postavami.</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>slider|kolko zospodu patri miereniu</t>
+          <t>slider|srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
         </is>
       </c>
     </row>
@@ -4783,27 +4783,27 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>SRDIECKA A TIENE</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>MIERIT OD POSTAVY</t>
+          <t>tien pod postavami: sila (0 = vypnuty)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>Mierenie zacina od postavy.</t>
+          <t>Sila tiena (odladene 0,3).</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -4813,7 +4813,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>switch|MIERIT OD POSTAVY</t>
+          <t>slider|tien pod postavami: sila (0 = vypnuty)</t>
         </is>
       </c>
     </row>
@@ -4825,27 +4825,27 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>ZONA PRE LAVY PALEC</t>
+          <t>SRDIECKA A TIENE</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>VOLNY POHYB (bez skoku)</t>
+          <t>tien pod postavami: velkost (x)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>Hrdina nechodi skokom k prstu.</t>
+          <t>Velkost tiena (odladene 1).</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -4855,7 +4855,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>switch|VOLNY POHYB (bez skoku)</t>
+          <t>slider|tien pod postavami: velkost (x)</t>
         </is>
       </c>
     </row>
@@ -4872,38 +4872,206 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>sirka</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>Sirka zony pre lavy palec.</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>slider|sirka</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>S106</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>slider</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>kolko zospodu patri miereniu</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>0.16</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>Spodna cast zony patri miereniu.</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>slider|kolko zospodu patri miereniu</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>S107</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
           <t>switch</t>
         </is>
       </c>
-      <c r="D106" s="2" t="inlineStr">
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>MIERIT OD POSTAVY</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>ZAP</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>Mierenie zacina od postavy.</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>switch|MIERIT OD POSTAVY</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>S108</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>switch</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>VOLNY POHYB (bez skoku)</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>ZAP</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>Hrdina nechodi skokom k prstu.</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>switch|VOLNY POHYB (bez skoku)</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>S109</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>ZONA PRE LAVY PALEC</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>switch</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
         <is>
           <t>POHYB KOPIRUJE PALEC</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr">
+      <c r="E110" t="inlineStr">
         <is>
           <t>VYP</t>
         </is>
       </c>
-      <c r="F106" s="2" t="inlineStr">
+      <c r="F110" s="2" t="inlineStr">
         <is>
           <t>Hrdina kopiruje pohyb palca.</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr">
+      <c r="G110" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr">
+      <c r="H110" t="inlineStr">
         <is>
           <t>switch|POHYB KOPIRUJE PALEC</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G106"/>
-  <conditionalFormatting sqref="G2:G106">
+  <autoFilter ref="A1:G110"/>
+  <conditionalFormatting sqref="G2:G110">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"A"</formula>
     </cfRule>
@@ -4912,7 +5080,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G110" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"A,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Package 3: reject warning blink and synthesised warning sounds (Pavel's phone test); keep only the 0.4 s brute wind-up before the grab
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014j5P4SqpYW49SirSP3JAGF
</commit_message>
<xml_diff>
--- a/PANEL_prvky.xlsx
+++ b/PANEL_prvky.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Panel'!$A$1:$G$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Panel'!$A$1:$G$108</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H110"/>
+  <dimension ref="A1:H108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>VAROVANIE PRED UTOKOM (blikanie)</t>
+          <t>ZVUK VAROVANIA OBORA</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Nepriatel pred utokom (udrer bezca, vystrel strelca, chytenie obora) blika do cervena.</t>
+          <t>Obor zavrci pred chytenim (zatial ticho, kym nie su hlasy).</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2637,7 +2637,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>switch|VAROVANIE PRED UTOKOM (blikanie)</t>
+          <t>switch|ZVUK VAROVANIA OBORA</t>
         </is>
       </c>
     </row>
@@ -2654,22 +2654,22 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>ZVUK VAROVANIA</t>
+          <t>obor: vymah pred chytenim (s)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Kazdy typ nepriatela zahra svoj zvuk na zaciatku utoku (zatial dockovy syntetizovany zvuk).</t>
+          <t>Obor sa pred chytenim na chvilu zastavi; vtedy mozes uhnut (0 = chyti okamzite).</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>switch|ZVUK VAROVANIA</t>
+          <t>slider|obor: vymah pred chytenim (s)</t>
         </is>
       </c>
     </row>
@@ -2696,22 +2696,18 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>button</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>varovanie: sila blikania</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
+          <t>TEST VIBRACIE (rovnaka ako pri mojom zasahu)</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Ako vyrazne nepriatel blika pred utokom (1 = plne).</t>
+          <t>Tlacidlo: jedna vibracia presne taka, ako pri tvojom zasahu (na zistenie, ci telefon vibruje).</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2721,7 +2717,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>slider|varovanie: sila blikania</t>
+          <t>button|TEST VIBRACIE (rovnaka ako pri mojom zasahu)</t>
         </is>
       </c>
     </row>
@@ -2738,22 +2734,22 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>obor: vymah pred chytenim (s)</t>
+          <t>CISLA POSKODENIA</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Obor sa pred chytenim zastavi, zavrci a blika; vtedy mozes uhnut (0 = chyti okamzite).</t>
+          <t>Nad zasiahnutym nepriatelom vyleti cislo poskodenia.</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2763,7 +2759,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>slider|obor: vymah pred chytenim (s)</t>
+          <t>switch|CISLA POSKODENIA</t>
         </is>
       </c>
     </row>
@@ -2780,18 +2776,22 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>TEST VIBRACIE (rovnaka ako pri mojom zasahu)</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr"/>
+          <t>velkost cisel poskodenia</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Tlacidlo: jedna vibracia presne taka, ako pri tvojom zasahu (na zistenie, ci telefon vibruje).</t>
+          <t>Velkost pisma cisel poskodenia.</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>button|TEST VIBRACIE (rovnaka ako pri mojom zasahu)</t>
+          <t>slider|velkost cisel poskodenia</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2823,7 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>CISLA POSKODENIA</t>
+          <t>KRITICKY ZASAH</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2833,7 +2833,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Nad zasiahnutym nepriatelom vyleti cislo poskodenia.</t>
+          <t>Cast zasahov je kritickych (2 zivoty, zlte cislo, silnejsie efekty).</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>switch|CISLA POSKODENIA</t>
+          <t>switch|KRITICKY ZASAH</t>
         </is>
       </c>
     </row>
@@ -2865,17 +2865,17 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>velkost cisel poskodenia</t>
+          <t>sanca na kriticky zasah (%)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Velkost pisma cisel poskodenia.</t>
+          <t>Kolko percent zasahov je kritickych (100 = vzdy na test).</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>slider|velkost cisel poskodenia</t>
+          <t>slider|sanca na kriticky zasah (%)</t>
         </is>
       </c>
     </row>
@@ -2907,17 +2907,17 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>KRITICKY ZASAH</t>
+          <t>HUDBA</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Cast zasahov je kritickych (2 zivoty, zlte cislo, silnejsie efekty).</t>
+          <t>Zapne/vypne hudbu.</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2927,7 +2927,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>switch|KRITICKY ZASAH</t>
+          <t>switch|HUDBA</t>
         </is>
       </c>
     </row>
@@ -2949,27 +2949,27 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>sanca na kriticky zasah (%)</t>
+          <t>hlasitost hudby (dB)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>15.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Kolko percent zasahov je kritickych (100 = vzdy na test).</t>
+          <t>Hlasitost hudby.</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>slider|sanca na kriticky zasah (%)</t>
+          <t>slider|hlasitost hudby (dB)</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>HUDBA</t>
+          <t>ZMRAZIT SVET (hybe sa len hrdina)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Zapne/vypne hudbu.</t>
+          <t>Zastavi nepriatelov, kotly a ich strely; hybe sa len hrdina.</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>switch|HUDBA</t>
+          <t>switch|ZMRAZIT SVET (hybe sa len hrdina)</t>
         </is>
       </c>
     </row>
@@ -3028,32 +3028,32 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>hlasitost hudby (dB)</t>
+          <t>VYPNUT BEZCOV</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Hlasitost hudby.</t>
+          <t>Nebudu sa objavovat bezci.</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>slider|hlasitost hudby (dB)</t>
+          <t>switch|VYPNUT BEZCOV</t>
         </is>
       </c>
     </row>
@@ -3075,7 +3075,7 @@
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>ZMRAZIT SVET (hybe sa len hrdina)</t>
+          <t>VYPNUT STRELCOV</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3085,7 +3085,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Zastavi nepriatelov, kotly a ich strely; hybe sa len hrdina.</t>
+          <t>Nebudu sa objavovat strelci.</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>switch|ZMRAZIT SVET (hybe sa len hrdina)</t>
+          <t>switch|VYPNUT STRELCOV</t>
         </is>
       </c>
     </row>
@@ -3117,17 +3117,17 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT BEZCOV</t>
+          <t>VYPNUT TUCNAKOV</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat bezci.</t>
+          <t>Nebudu sa objavovat tucniaci.</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3137,7 +3137,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>switch|VYPNUT BEZCOV</t>
+          <t>switch|VYPNUT TUCNAKOV</t>
         </is>
       </c>
     </row>
@@ -3154,22 +3154,22 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT STRELCOV</t>
+          <t>kolko bezcov naraz (test)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat strelci.</t>
+          <t>Kolko bezcov je naraz v hre.</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3179,7 +3179,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>switch|VYPNUT STRELCOV</t>
+          <t>slider|kolko bezcov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -3196,22 +3196,22 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT TUCNAKOV</t>
+          <t>kolko strelcov naraz (test)</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat tucniaci.</t>
+          <t>Kolko strelcov je naraz v hre.</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3221,7 +3221,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>switch|VYPNUT TUCNAKOV</t>
+          <t>slider|kolko strelcov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -3243,17 +3243,17 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>kolko bezcov naraz (test)</t>
+          <t>kolko tucnakov naraz (test)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Kolko bezcov je naraz v hre.</t>
+          <t>Kolko tucniakov je naraz v hre.</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>slider|kolko bezcov naraz (test)</t>
+          <t>slider|kolko tucnakov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>TEST</t>
+          <t>POHYB</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3285,17 +3285,17 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>kolko strelcov naraz (test)</t>
+          <t>posun palca pre plnu rychlost vlavo</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Kolko strelcov je naraz v hre.</t>
+          <t>Ako daleko od stredu paky treba posunut palec pre plnu rychlost (mensie cislo = rychlejsie plna rychlost, kratsia pomala zona).</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3305,7 +3305,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>slider|kolko strelcov naraz (test)</t>
+          <t>slider|posun palca pre plnu rychlost vlavo</t>
         </is>
       </c>
     </row>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>TEST</t>
+          <t>POHYB</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3327,17 +3327,17 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>kolko tucnakov naraz (test)</t>
+          <t>posun palca pre plnu rychlost vpravo</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Kolko tucniakov je naraz v hre.</t>
+          <t>To iste, vpravo; plati aj pre pohyb hore a dole.</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>slider|kolko tucnakov naraz (test)</t>
+          <t>slider|posun palca pre plnu rychlost vpravo</t>
         </is>
       </c>
     </row>
@@ -3369,17 +3369,17 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>posun palca pre plnu rychlost vlavo</t>
+          <t>o kolko pomalsi je pohyb hore-dole</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Ako daleko od stredu paky treba posunut palec pre plnu rychlost (mensie cislo = rychlejsie plna rychlost, kratsia pomala zona).</t>
+          <t>1 = hore/dole rovnako rychlo ako do stran; menej = pomalsie.</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -3389,7 +3389,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>slider|posun palca pre plnu rychlost vlavo</t>
+          <t>slider|o kolko pomalsi je pohyb hore-dole</t>
         </is>
       </c>
     </row>
@@ -3401,7 +3401,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>POHYB</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3411,27 +3411,27 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>posun palca pre plnu rychlost vpravo</t>
+          <t>ako blizko k postave prestane mierit</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>15.0</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>To iste, vpravo; plati aj pre pohyb hore a dole.</t>
+          <t>Mierenie sa vypne, ked je palec blizko postavy.</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>slider|posun palca pre plnu rychlost vpravo</t>
+          <t>slider|ako blizko k postave prestane mierit</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>POHYB</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>o kolko pomalsi je pohyb hore-dole</t>
+          <t>rychlost postavy</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3463,7 +3463,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>1 = hore/dole rovnako rychlo ako do stran; menej = pomalsie.</t>
+          <t>Nasobok rychlosti hrdinu.</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3473,7 +3473,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>slider|o kolko pomalsi je pohyb hore-dole</t>
+          <t>slider|rychlost postavy</t>
         </is>
       </c>
     </row>
@@ -3495,17 +3495,17 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>ako blizko k postave prestane mierit</t>
+          <t>pohyb pocas hodu (0 = stoji)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Mierenie sa vypne, ked je palec blizko postavy.</t>
+          <t>Ako rychlo sa hrdina hybe pocas hodu.</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>slider|ako blizko k postave prestane mierit</t>
+          <t>slider|pohyb pocas hodu (0 = stoji)</t>
         </is>
       </c>
     </row>
@@ -3537,27 +3537,27 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>rychlost postavy</t>
+          <t>rychlost zamachu pri hode (1 = povodna)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti hrdinu.</t>
+          <t>Rychlost animacie hodu.</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>slider|rychlost postavy</t>
+          <t>slider|rychlost zamachu pri hode (1 = povodna)</t>
         </is>
       </c>
     </row>
@@ -3574,22 +3574,22 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>pohyb pocas hodu (0 = stoji)</t>
+          <t>HRDINA 2x (vypnute = 1x)</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Ako rychlo sa hrdina hybe pocas hodu.</t>
+          <t>Velkost hrdinu.</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3599,7 +3599,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>slider|pohyb pocas hodu (0 = stoji)</t>
+          <t>switch|HRDINA 2x (vypnute = 1x)</t>
         </is>
       </c>
     </row>
@@ -3616,32 +3616,32 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>rychlost zamachu pri hode (1 = povodna)</t>
+          <t>SEKERA (vypnute = gulky)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Rychlost animacie hodu.</t>
+          <t>Prepina zbran: sekera alebo gulky.</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>slider|rychlost zamachu pri hode (1 = povodna)</t>
+          <t>switch|SEKERA (vypnute = gulky)</t>
         </is>
       </c>
     </row>
@@ -3658,32 +3658,32 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>HRDINA 2x (vypnute = 1x)</t>
+          <t>dosah sekery</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>350.0</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Velkost hrdinu.</t>
+          <t>Ako daleko sekera doletí.</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>switch|HRDINA 2x (vypnute = 1x)</t>
+          <t>slider|dosah sekery</t>
         </is>
       </c>
     </row>
@@ -3700,22 +3700,22 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>SEKERA (vypnute = gulky)</t>
+          <t>rychlost sekery</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>650.0</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Prepina zbran: sekera alebo gulky.</t>
+          <t>Rychlost sekery smerom k cielu (spat je 1,5x).</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3725,7 +3725,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>switch|SEKERA (vypnute = gulky)</t>
+          <t>slider|rychlost sekery</t>
         </is>
       </c>
     </row>
@@ -3742,22 +3742,18 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>button</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>dosah sekery</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>350.0</t>
-        </is>
-      </c>
+          <t>NOVE SUDY (postavi ich pred hrdinu)</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Ako daleko sekera doletí.</t>
+          <t>Tlacidlo: znova postavi sudy.</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3767,7 +3763,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>slider|dosah sekery</t>
+          <t>button|NOVE SUDY (postavi ich pred hrdinu)</t>
         </is>
       </c>
     </row>
@@ -3789,27 +3785,27 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>rychlost sekery</t>
+          <t>aky vysoky kus tela hraca sa da trafit (0-1)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>650.0</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Rychlost sekery smerom k cielu (spat je 1,5x).</t>
+          <t>Vyska zasiahnutelnej casti hrdinu.</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>slider|rychlost sekery</t>
+          <t>slider|aky vysoky kus tela hraca sa da trafit (0-1)</t>
         </is>
       </c>
     </row>
@@ -3821,23 +3817,27 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>NOVE SUDY (postavi ich pred hrdinu)</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr"/>
+          <t>rychlost bezcov</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Tlacidlo: znova postavi sudy.</t>
+          <t>Nasobok rychlosti bezcov.</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -3847,7 +3847,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>button|NOVE SUDY (postavi ich pred hrdinu)</t>
+          <t>slider|rychlost bezcov</t>
         </is>
       </c>
     </row>
@@ -3859,7 +3859,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3869,27 +3869,27 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>aky vysoky kus tela hraca sa da trafit (0-1)</t>
+          <t>rychlost strelcov</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Vyska zasiahnutelnej casti hrdinu.</t>
+          <t>Nasobok rychlosti strelcov.</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>slider|aky vysoky kus tela hraca sa da trafit (0-1)</t>
+          <t>slider|rychlost strelcov</t>
         </is>
       </c>
     </row>
@@ -3911,27 +3911,27 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>rychlost bezcov</t>
+          <t>na aku vzdialenost si bezec vsimne hraca (px)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>640.0</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti bezcov.</t>
+          <t>Dosah, od ktoreho bezec zacne prenasledovat.</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>slider|rychlost bezcov</t>
+          <t>slider|na aku vzdialenost si bezec vsimne hraca (px)</t>
         </is>
       </c>
     </row>
@@ -3948,22 +3948,22 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>rychlost strelcov</t>
+          <t>UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti strelcov.</t>
+          <t>Nakresli kruh sekery a obdlzniky zasahu nepriatelov a hrdinu.</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -3973,7 +3973,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>slider|rychlost strelcov</t>
+          <t>switch|UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
         </is>
       </c>
     </row>
@@ -3995,27 +3995,27 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>na aku vzdialenost si bezec vsimne hraca (px)</t>
+          <t>sekera: polomer zasahu (px)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>640.0</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Dosah, od ktoreho bezec zacne prenasledovat.</t>
+          <t>Velkost kruhu sekery; sekera zasiahne kazdeho, koho obdlznik sa dotkne kruhu.</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>slider|na aku vzdialenost si bezec vsimne hraca (px)</t>
+          <t>slider|sekera: polomer zasahu (px)</t>
         </is>
       </c>
     </row>
@@ -4037,7 +4037,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
+          <t>UKAZ ZONU UDERU BEZCA</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4047,17 +4047,17 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Nakresli kruh sekery a obdlzniky zasahu nepriatelov a hrdinu.</t>
+          <t>Nakresli kruh, kam dopadne uder bezca.</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>switch|UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
+          <t>switch|UKAZ ZONU UDERU BEZCA</t>
         </is>
       </c>
     </row>
@@ -4079,27 +4079,27 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>sekera: polomer zasahu (px)</t>
+          <t>zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Velkost kruhu sekery; sekera zasiahne kazdeho, koho obdlznik sa dotkne kruhu.</t>
+          <t>Poloha zony uderu.</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>slider|sekera: polomer zasahu (px)</t>
+          <t>slider|zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
         </is>
       </c>
     </row>
@@ -4116,22 +4116,22 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>UKAZ ZONU UDERU BEZCA</t>
+          <t>zona uderu: vyska dopadu nad nohami bezca (px)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Nakresli kruh, kam dopadne uder bezca.</t>
+          <t>Poloha zony uderu.</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -4141,7 +4141,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>switch|UKAZ ZONU UDERU BEZCA</t>
+          <t>slider|zona uderu: vyska dopadu nad nohami bezca (px)</t>
         </is>
       </c>
     </row>
@@ -4163,7 +4163,7 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
+          <t>zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -4173,7 +4173,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>Poloha zony uderu.</t>
+          <t>Velkost zony uderu.</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>slider|zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
+          <t>slider|zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
         </is>
       </c>
     </row>
@@ -4205,17 +4205,17 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: vyska dopadu nad nohami bezca (px)</t>
+          <t>kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>Poloha zony uderu.</t>
+          <t>Casovanie zasahu v animacii.</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -4225,7 +4225,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>slider|zona uderu: vyska dopadu nad nohami bezca (px)</t>
+          <t>slider|kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
         </is>
       </c>
     </row>
@@ -4247,17 +4247,17 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
+          <t>aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>Velkost zony uderu.</t>
+          <t>Vyska zasiahnutelnej casti nepriatela.</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>slider|zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
+          <t>slider|aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
         </is>
       </c>
     </row>
@@ -4284,32 +4284,32 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
+          <t>PEVNE TELA (nikto cez nikoho neprejde)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>Casovanie zasahu v animacii.</t>
+          <t>Zapne pevne nohy postav; nikto cez nikoho neprejde.</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>slider|kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
+          <t>switch|PEVNE TELA (nikto cez nikoho neprejde)</t>
         </is>
       </c>
     </row>
@@ -4331,17 +4331,17 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
+          <t>pevne telo: hlbka nohy (px; 54 = cele telo)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>Vyska zasiahnutelnej casti nepriatela.</t>
+          <t>Hlbka pevneho tela (odladene 30).</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -4351,7 +4351,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>slider|aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
+          <t>slider|pevne telo: hlbka nohy (px; 54 = cele telo)</t>
         </is>
       </c>
     </row>
@@ -4368,32 +4368,32 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>PEVNE TELA (nikto cez nikoho neprejde)</t>
+          <t>pevne telo: sirka nohy (px)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>Zapne pevne nohy postav; nikto cez nikoho neprejde.</t>
+          <t>Sirka pevneho tela (odladene 60).</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>switch|PEVNE TELA (nikto cez nikoho neprejde)</t>
+          <t>slider|pevne telo: sirka nohy (px)</t>
         </is>
       </c>
     </row>
@@ -4415,17 +4415,17 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>pevne telo: hlbka nohy (px; 54 = cele telo)</t>
+          <t>ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>Hlbka pevneho tela (odladene 30).</t>
+          <t>Stary mak odtlacania; funguje len ked su PEVNE TELA vypnute.</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -4435,7 +4435,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>slider|pevne telo: hlbka nohy (px; 54 = cele telo)</t>
+          <t>slider|ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
         </is>
       </c>
     </row>
@@ -4447,7 +4447,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>ODHODENIE PO ZASAHU</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -4457,27 +4457,27 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>pevne telo: sirka nohy (px)</t>
+          <t>bezec odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>90.0</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Sirka pevneho tela (odladene 60).</t>
+          <t>Dlzka odhodenia hrdinu po zasahu bezca.</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>slider|pevne telo: sirka nohy (px)</t>
+          <t>slider|bezec odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -4489,7 +4489,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>ODHODENIE PO ZASAHU</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -4499,27 +4499,27 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
+          <t>strela strelca odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>Stary mak odtlacania; funguje len ked su PEVNE TELA vypnute.</t>
+          <t>Dlzka odhodenia hrdinu po zasahu strely.</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>slider|ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
+          <t>slider|strela strelca odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -4541,17 +4541,17 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>bezec odhodi hrdinu (px)</t>
+          <t>sekera odhodi nepriatela (px)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu po zasahu bezca.</t>
+          <t>Dlzka odhodenia nepriatela po zasahu sekery.</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -4561,7 +4561,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>slider|bezec odhodi hrdinu (px)</t>
+          <t>slider|sekera odhodi nepriatela (px)</t>
         </is>
       </c>
     </row>
@@ -4583,17 +4583,17 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>strela strelca odhodi hrdinu (px)</t>
+          <t>vybuch kotla odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>140.0</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu po zasahu strely.</t>
+          <t>Dlzka odhodenia hrdinu pri vybuchu kotla.</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -4603,7 +4603,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>slider|strela strelca odhodi hrdinu (px)</t>
+          <t>slider|vybuch kotla odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -4625,27 +4625,27 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>sekera odhodi nepriatela (px)</t>
+          <t>odhodenie: ako dlho trva (s)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia nepriatela po zasahu sekery.</t>
+          <t>Trvanie odhodenia (odladene 0,4).</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>slider|sekera odhodi nepriatela (px)</t>
+          <t>slider|odhodenie: ako dlho trva (s)</t>
         </is>
       </c>
     </row>
@@ -4657,7 +4657,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>SRDIECKA A TIENE</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -4667,17 +4667,17 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>vybuch kotla odhodi hrdinu (px)</t>
+          <t>srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>140.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu pri vybuchu kotla.</t>
+          <t>Zivoty nad postavami.</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -4687,7 +4687,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>slider|vybuch kotla odhodi hrdinu (px)</t>
+          <t>slider|srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
         </is>
       </c>
     </row>
@@ -4699,7 +4699,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>SRDIECKA A TIENE</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -4709,17 +4709,17 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>odhodenie: ako dlho trva (s)</t>
+          <t>tien pod postavami: sila (0 = vypnuty)</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>Trvanie odhodenia (odladene 0,4).</t>
+          <t>Sila tiena (odladene 0,3).</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -4729,7 +4729,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>slider|odhodenie: ako dlho trva (s)</t>
+          <t>slider|tien pod postavami: sila (0 = vypnuty)</t>
         </is>
       </c>
     </row>
@@ -4751,27 +4751,27 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+          <t>tien pod postavami: velkost (x)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>Zivoty nad postavami.</t>
+          <t>Velkost tiena (odladene 1).</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>slider|srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+          <t>slider|tien pod postavami: velkost (x)</t>
         </is>
       </c>
     </row>
@@ -4783,7 +4783,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>ZONA PRE LAVY PALEC</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -4793,17 +4793,17 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>tien pod postavami: sila (0 = vypnuty)</t>
+          <t>sirka</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>Sila tiena (odladene 0,3).</t>
+          <t>Sirka zony pre lavy palec.</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -4813,7 +4813,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>slider|tien pod postavami: sila (0 = vypnuty)</t>
+          <t>slider|sirka</t>
         </is>
       </c>
     </row>
@@ -4825,7 +4825,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>ZONA PRE LAVY PALEC</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -4835,17 +4835,17 @@
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>tien pod postavami: velkost (x)</t>
+          <t>kolko zospodu patri miereniu</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.16</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>Velkost tiena (odladene 1).</t>
+          <t>Spodna cast zony patri miereniu.</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -4855,7 +4855,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>slider|tien pod postavami: velkost (x)</t>
+          <t>slider|kolko zospodu patri miereniu</t>
         </is>
       </c>
     </row>
@@ -4872,22 +4872,22 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>sirka</t>
+          <t>MIERIT OD POSTAVY</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>Sirka zony pre lavy palec.</t>
+          <t>Mierenie zacina od postavy.</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -4897,7 +4897,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>slider|sirka</t>
+          <t>switch|MIERIT OD POSTAVY</t>
         </is>
       </c>
     </row>
@@ -4914,22 +4914,22 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>kolko zospodu patri miereniu</t>
+          <t>VOLNY POHYB (bez skoku)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>Spodna cast zony patri miereniu.</t>
+          <t>Hrdina nechodi skokom k prstu.</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -4939,7 +4939,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>slider|kolko zospodu patri miereniu</t>
+          <t>switch|VOLNY POHYB (bez skoku)</t>
         </is>
       </c>
     </row>
@@ -4961,17 +4961,17 @@
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>MIERIT OD POSTAVY</t>
+          <t>POHYB KOPIRUJE PALEC</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>Mierenie zacina od postavy.</t>
+          <t>Hrdina kopiruje pohyb palca.</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -4981,97 +4981,13 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>switch|MIERIT OD POSTAVY</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
-        <is>
-          <t>S108</t>
-        </is>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>ZONA PRE LAVY PALEC</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>switch</t>
-        </is>
-      </c>
-      <c r="D109" s="2" t="inlineStr">
-        <is>
-          <t>VOLNY POHYB (bez skoku)</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>ZAP</t>
-        </is>
-      </c>
-      <c r="F109" s="2" t="inlineStr">
-        <is>
-          <t>Hrdina nechodi skokom k prstu.</t>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H109" t="inlineStr">
-        <is>
-          <t>switch|VOLNY POHYB (bez skoku)</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
-        <is>
-          <t>S109</t>
-        </is>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>ZONA PRE LAVY PALEC</t>
-        </is>
-      </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>switch</t>
-        </is>
-      </c>
-      <c r="D110" s="2" t="inlineStr">
-        <is>
-          <t>POHYB KOPIRUJE PALEC</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>VYP</t>
-        </is>
-      </c>
-      <c r="F110" s="2" t="inlineStr">
-        <is>
-          <t>Hrdina kopiruje pohyb palca.</t>
-        </is>
-      </c>
-      <c r="G110" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H110" t="inlineStr">
-        <is>
           <t>switch|POHYB KOPIRUJE PALEC</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G110"/>
-  <conditionalFormatting sqref="G2:G110">
+  <autoFilter ref="A1:G108"/>
+  <conditionalFormatting sqref="G2:G108">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"A"</formula>
     </cfRule>
@@ -5080,7 +4996,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G110" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G108" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"A,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Close package 3: warning blink and brute wind-up rejected and removed, dirt variants kept; archive F2, D4 postponed; package 4 is next. Restores CRLF line endings of tuning.gd and debug_overlay.gd
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014j5P4SqpYW49SirSP3JAGF
</commit_message>
<xml_diff>
--- a/PANEL_prvky.xlsx
+++ b/PANEL_prvky.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Panel'!$A$1:$G$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Panel'!$A$1:$G$106</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H108"/>
+  <dimension ref="A1:H106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2612,22 +2612,18 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>button</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>ZVUK VAROVANIA OBORA</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>ZAP</t>
-        </is>
-      </c>
+          <t>TEST VIBRACIE (rovnaka ako pri mojom zasahu)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Obor zavrci pred chytenim (zatial ticho, kym nie su hlasy).</t>
+          <t>Tlacidlo: jedna vibracia presne taka, ako pri tvojom zasahu (na zistenie, ci telefon vibruje).</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2637,7 +2633,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>switch|ZVUK VAROVANIA OBORA</t>
+          <t>button|TEST VIBRACIE (rovnaka ako pri mojom zasahu)</t>
         </is>
       </c>
     </row>
@@ -2654,22 +2650,22 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>obor: vymah pred chytenim (s)</t>
+          <t>CISLA POSKODENIA</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Obor sa pred chytenim na chvilu zastavi; vtedy mozes uhnut (0 = chyti okamzite).</t>
+          <t>Nad zasiahnutym nepriatelom vyleti cislo poskodenia.</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2679,7 +2675,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>slider|obor: vymah pred chytenim (s)</t>
+          <t>switch|CISLA POSKODENIA</t>
         </is>
       </c>
     </row>
@@ -2696,18 +2692,22 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>TEST VIBRACIE (rovnaka ako pri mojom zasahu)</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr"/>
+          <t>velkost cisel poskodenia</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>16.0</t>
+        </is>
+      </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Tlacidlo: jedna vibracia presne taka, ako pri tvojom zasahu (na zistenie, ci telefon vibruje).</t>
+          <t>Velkost pisma cisel poskodenia.</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2717,7 +2717,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>button|TEST VIBRACIE (rovnaka ako pri mojom zasahu)</t>
+          <t>slider|velkost cisel poskodenia</t>
         </is>
       </c>
     </row>
@@ -2739,7 +2739,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>CISLA POSKODENIA</t>
+          <t>KRITICKY ZASAH</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Nad zasiahnutym nepriatelom vyleti cislo poskodenia.</t>
+          <t>Cast zasahov je kritickych (2 zivoty, zlte cislo, silnejsie efekty).</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>switch|CISLA POSKODENIA</t>
+          <t>switch|KRITICKY ZASAH</t>
         </is>
       </c>
     </row>
@@ -2781,17 +2781,17 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>velkost cisel poskodenia</t>
+          <t>sanca na kriticky zasah (%)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>16.0</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>Velkost pisma cisel poskodenia.</t>
+          <t>Kolko percent zasahov je kritickych (100 = vzdy na test).</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>slider|velkost cisel poskodenia</t>
+          <t>slider|sanca na kriticky zasah (%)</t>
         </is>
       </c>
     </row>
@@ -2823,17 +2823,17 @@
       </c>
       <c r="D57" s="2" t="inlineStr">
         <is>
-          <t>KRITICKY ZASAH</t>
+          <t>HUDBA</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>Cast zasahov je kritickych (2 zivoty, zlte cislo, silnejsie efekty).</t>
+          <t>Zapne/vypne hudbu.</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>switch|KRITICKY ZASAH</t>
+          <t>switch|HUDBA</t>
         </is>
       </c>
     </row>
@@ -2865,27 +2865,27 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>sanca na kriticky zasah (%)</t>
+          <t>hlasitost hudby (dB)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>15.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Kolko percent zasahov je kritickych (100 = vzdy na test).</t>
+          <t>Hlasitost hudby.</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>slider|sanca na kriticky zasah (%)</t>
+          <t>slider|hlasitost hudby (dB)</t>
         </is>
       </c>
     </row>
@@ -2907,7 +2907,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>HUDBA</t>
+          <t>ZMRAZIT SVET (hybe sa len hrdina)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2917,7 +2917,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>Zapne/vypne hudbu.</t>
+          <t>Zastavi nepriatelov, kotly a ich strely; hybe sa len hrdina.</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -2927,7 +2927,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>switch|HUDBA</t>
+          <t>switch|ZMRAZIT SVET (hybe sa len hrdina)</t>
         </is>
       </c>
     </row>
@@ -2944,32 +2944,32 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>hlasitost hudby (dB)</t>
+          <t>VYPNUT BEZCOV</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>Hlasitost hudby.</t>
+          <t>Nebudu sa objavovat bezci.</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>slider|hlasitost hudby (dB)</t>
+          <t>switch|VYPNUT BEZCOV</t>
         </is>
       </c>
     </row>
@@ -2991,7 +2991,7 @@
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>ZMRAZIT SVET (hybe sa len hrdina)</t>
+          <t>VYPNUT STRELCOV</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3001,7 +3001,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Zastavi nepriatelov, kotly a ich strely; hybe sa len hrdina.</t>
+          <t>Nebudu sa objavovat strelci.</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3011,7 +3011,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>switch|ZMRAZIT SVET (hybe sa len hrdina)</t>
+          <t>switch|VYPNUT STRELCOV</t>
         </is>
       </c>
     </row>
@@ -3033,17 +3033,17 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT BEZCOV</t>
+          <t>VYPNUT TUCNAKOV</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat bezci.</t>
+          <t>Nebudu sa objavovat tucniaci.</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3053,7 +3053,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>switch|VYPNUT BEZCOV</t>
+          <t>switch|VYPNUT TUCNAKOV</t>
         </is>
       </c>
     </row>
@@ -3070,22 +3070,22 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT STRELCOV</t>
+          <t>kolko bezcov naraz (test)</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat strelci.</t>
+          <t>Kolko bezcov je naraz v hre.</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>switch|VYPNUT STRELCOV</t>
+          <t>slider|kolko bezcov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -3112,22 +3112,22 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>VYPNUT TUCNAKOV</t>
+          <t>kolko strelcov naraz (test)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Nebudu sa objavovat tucniaci.</t>
+          <t>Kolko strelcov je naraz v hre.</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3137,7 +3137,7 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>switch|VYPNUT TUCNAKOV</t>
+          <t>slider|kolko strelcov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -3159,17 +3159,17 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>kolko bezcov naraz (test)</t>
+          <t>kolko tucnakov naraz (test)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Kolko bezcov je naraz v hre.</t>
+          <t>Kolko tucniakov je naraz v hre.</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3179,7 +3179,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>slider|kolko bezcov naraz (test)</t>
+          <t>slider|kolko tucnakov naraz (test)</t>
         </is>
       </c>
     </row>
@@ -3191,7 +3191,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>TEST</t>
+          <t>POHYB</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3201,17 +3201,17 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>kolko strelcov naraz (test)</t>
+          <t>posun palca pre plnu rychlost vlavo</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Kolko strelcov je naraz v hre.</t>
+          <t>Ako daleko od stredu paky treba posunut palec pre plnu rychlost (mensie cislo = rychlejsie plna rychlost, kratsia pomala zona).</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3221,7 +3221,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>slider|kolko strelcov naraz (test)</t>
+          <t>slider|posun palca pre plnu rychlost vlavo</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3233,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>TEST</t>
+          <t>POHYB</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3243,17 +3243,17 @@
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>kolko tucnakov naraz (test)</t>
+          <t>posun palca pre plnu rychlost vpravo</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>15.0</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Kolko tucniakov je naraz v hre.</t>
+          <t>To iste, vpravo; plati aj pre pohyb hore a dole.</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3263,7 +3263,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>slider|kolko tucnakov naraz (test)</t>
+          <t>slider|posun palca pre plnu rychlost vpravo</t>
         </is>
       </c>
     </row>
@@ -3285,17 +3285,17 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>posun palca pre plnu rychlost vlavo</t>
+          <t>o kolko pomalsi je pohyb hore-dole</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Ako daleko od stredu paky treba posunut palec pre plnu rychlost (mensie cislo = rychlejsie plna rychlost, kratsia pomala zona).</t>
+          <t>1 = hore/dole rovnako rychlo ako do stran; menej = pomalsie.</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3305,7 +3305,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>slider|posun palca pre plnu rychlost vlavo</t>
+          <t>slider|o kolko pomalsi je pohyb hore-dole</t>
         </is>
       </c>
     </row>
@@ -3317,7 +3317,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>POHYB</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3327,27 +3327,27 @@
       </c>
       <c r="D69" s="2" t="inlineStr">
         <is>
-          <t>posun palca pre plnu rychlost vpravo</t>
+          <t>ako blizko k postave prestane mierit</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>15.0</t>
+          <t>9.0</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>To iste, vpravo; plati aj pre pohyb hore a dole.</t>
+          <t>Mierenie sa vypne, ked je palec blizko postavy.</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>slider|posun palca pre plnu rychlost vpravo</t>
+          <t>slider|ako blizko k postave prestane mierit</t>
         </is>
       </c>
     </row>
@@ -3359,7 +3359,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>POHYB</t>
+          <t>MIERENIE</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3369,7 +3369,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>o kolko pomalsi je pohyb hore-dole</t>
+          <t>rychlost postavy</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3379,7 +3379,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>1 = hore/dole rovnako rychlo ako do stran; menej = pomalsie.</t>
+          <t>Nasobok rychlosti hrdinu.</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -3389,7 +3389,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>slider|o kolko pomalsi je pohyb hore-dole</t>
+          <t>slider|rychlost postavy</t>
         </is>
       </c>
     </row>
@@ -3411,17 +3411,17 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>ako blizko k postave prestane mierit</t>
+          <t>pohyb pocas hodu (0 = stoji)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>9.0</t>
+          <t>0.0</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Mierenie sa vypne, ked je palec blizko postavy.</t>
+          <t>Ako rychlo sa hrdina hybe pocas hodu.</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3431,7 +3431,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>slider|ako blizko k postave prestane mierit</t>
+          <t>slider|pohyb pocas hodu (0 = stoji)</t>
         </is>
       </c>
     </row>
@@ -3453,27 +3453,27 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>rychlost postavy</t>
+          <t>rychlost zamachu pri hode (1 = povodna)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti hrdinu.</t>
+          <t>Rychlost animacie hodu.</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>slider|rychlost postavy</t>
+          <t>slider|rychlost zamachu pri hode (1 = povodna)</t>
         </is>
       </c>
     </row>
@@ -3490,22 +3490,22 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>pohyb pocas hodu (0 = stoji)</t>
+          <t>HRDINA 2x (vypnute = 1x)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Ako rychlo sa hrdina hybe pocas hodu.</t>
+          <t>Velkost hrdinu.</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>slider|pohyb pocas hodu (0 = stoji)</t>
+          <t>switch|HRDINA 2x (vypnute = 1x)</t>
         </is>
       </c>
     </row>
@@ -3532,32 +3532,32 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>rychlost zamachu pri hode (1 = povodna)</t>
+          <t>SEKERA (vypnute = gulky)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Rychlost animacie hodu.</t>
+          <t>Prepina zbran: sekera alebo gulky.</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>slider|rychlost zamachu pri hode (1 = povodna)</t>
+          <t>switch|SEKERA (vypnute = gulky)</t>
         </is>
       </c>
     </row>
@@ -3574,32 +3574,32 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>HRDINA 2x (vypnute = 1x)</t>
+          <t>dosah sekery</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>350.0</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Velkost hrdinu.</t>
+          <t>Ako daleko sekera doletí.</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>switch|HRDINA 2x (vypnute = 1x)</t>
+          <t>slider|dosah sekery</t>
         </is>
       </c>
     </row>
@@ -3616,22 +3616,22 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>SEKERA (vypnute = gulky)</t>
+          <t>rychlost sekery</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>650.0</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Prepina zbran: sekera alebo gulky.</t>
+          <t>Rychlost sekery smerom k cielu (spat je 1,5x).</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3641,7 +3641,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>switch|SEKERA (vypnute = gulky)</t>
+          <t>slider|rychlost sekery</t>
         </is>
       </c>
     </row>
@@ -3658,22 +3658,18 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>button</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>dosah sekery</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>350.0</t>
-        </is>
-      </c>
+          <t>NOVE SUDY (postavi ich pred hrdinu)</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr"/>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Ako daleko sekera doletí.</t>
+          <t>Tlacidlo: znova postavi sudy.</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3683,7 +3679,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>slider|dosah sekery</t>
+          <t>button|NOVE SUDY (postavi ich pred hrdinu)</t>
         </is>
       </c>
     </row>
@@ -3705,27 +3701,27 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>rychlost sekery</t>
+          <t>aky vysoky kus tela hraca sa da trafit (0-1)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>650.0</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Rychlost sekery smerom k cielu (spat je 1,5x).</t>
+          <t>Vyska zasiahnutelnej casti hrdinu.</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>slider|rychlost sekery</t>
+          <t>slider|aky vysoky kus tela hraca sa da trafit (0-1)</t>
         </is>
       </c>
     </row>
@@ -3737,23 +3733,27 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>button</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>NOVE SUDY (postavi ich pred hrdinu)</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr"/>
+          <t>rychlost bezcov</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Tlacidlo: znova postavi sudy.</t>
+          <t>Nasobok rychlosti bezcov.</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>button|NOVE SUDY (postavi ich pred hrdinu)</t>
+          <t>slider|rychlost bezcov</t>
         </is>
       </c>
     </row>
@@ -3775,7 +3775,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>MIERENIE</t>
+          <t>NEPRIATELIA</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3785,27 +3785,27 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>aky vysoky kus tela hraca sa da trafit (0-1)</t>
+          <t>rychlost strelcov</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>Vyska zasiahnutelnej casti hrdinu.</t>
+          <t>Nasobok rychlosti strelcov.</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>slider|aky vysoky kus tela hraca sa da trafit (0-1)</t>
+          <t>slider|rychlost strelcov</t>
         </is>
       </c>
     </row>
@@ -3827,27 +3827,27 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>rychlost bezcov</t>
+          <t>na aku vzdialenost si bezec vsimne hraca (px)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>640.0</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti bezcov.</t>
+          <t>Dosah, od ktoreho bezec zacne prenasledovat.</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>slider|rychlost bezcov</t>
+          <t>slider|na aku vzdialenost si bezec vsimne hraca (px)</t>
         </is>
       </c>
     </row>
@@ -3864,22 +3864,22 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>rychlost strelcov</t>
+          <t>UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Nasobok rychlosti strelcov.</t>
+          <t>Nakresli kruh sekery a obdlzniky zasahu nepriatelov a hrdinu.</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -3889,7 +3889,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>slider|rychlost strelcov</t>
+          <t>switch|UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
         </is>
       </c>
     </row>
@@ -3911,27 +3911,27 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>na aku vzdialenost si bezec vsimne hraca (px)</t>
+          <t>sekera: polomer zasahu (px)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>640.0</t>
+          <t>20.0</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Dosah, od ktoreho bezec zacne prenasledovat.</t>
+          <t>Velkost kruhu sekery; sekera zasiahne kazdeho, koho obdlznik sa dotkne kruhu.</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>slider|na aku vzdialenost si bezec vsimne hraca (px)</t>
+          <t>slider|sekera: polomer zasahu (px)</t>
         </is>
       </c>
     </row>
@@ -3953,7 +3953,7 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
+          <t>UKAZ ZONU UDERU BEZCA</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3963,17 +3963,17 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Nakresli kruh sekery a obdlzniky zasahu nepriatelov a hrdinu.</t>
+          <t>Nakresli kruh, kam dopadne uder bezca.</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>switch|UKAZ ZONY ZASAHU (sekera, nepriatelia, hrdina)</t>
+          <t>switch|UKAZ ZONU UDERU BEZCA</t>
         </is>
       </c>
     </row>
@@ -3995,27 +3995,27 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>sekera: polomer zasahu (px)</t>
+          <t>zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>20.0</t>
+          <t>40.0</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Velkost kruhu sekery; sekera zasiahne kazdeho, koho obdlznik sa dotkne kruhu.</t>
+          <t>Poloha zony uderu.</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>slider|sekera: polomer zasahu (px)</t>
+          <t>slider|zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
         </is>
       </c>
     </row>
@@ -4032,22 +4032,22 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>UKAZ ZONU UDERU BEZCA</t>
+          <t>zona uderu: vyska dopadu nad nohami bezca (px)</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>VYP</t>
+          <t>50.0</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Nakresli kruh, kam dopadne uder bezca.</t>
+          <t>Poloha zony uderu.</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -4057,7 +4057,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>switch|UKAZ ZONU UDERU BEZCA</t>
+          <t>slider|zona uderu: vyska dopadu nad nohami bezca (px)</t>
         </is>
       </c>
     </row>
@@ -4079,7 +4079,7 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
+          <t>zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4089,7 +4089,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Poloha zony uderu.</t>
+          <t>Velkost zony uderu.</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -4099,7 +4099,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>slider|zona uderu: ako daleko pred bezcom dopadne zbran (px)</t>
+          <t>slider|zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
         </is>
       </c>
     </row>
@@ -4121,17 +4121,17 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: vyska dopadu nad nohami bezca (px)</t>
+          <t>kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>50.0</t>
+          <t>0.7</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Poloha zony uderu.</t>
+          <t>Casovanie zasahu v animacii.</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -4141,7 +4141,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>slider|zona uderu: vyska dopadu nad nohami bezca (px)</t>
+          <t>slider|kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
         </is>
       </c>
     </row>
@@ -4163,17 +4163,17 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
+          <t>aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>40.0</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>Velkost zony uderu.</t>
+          <t>Vyska zasiahnutelnej casti nepriatela.</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -4183,7 +4183,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>slider|zona uderu: polomer kruhu okolo miesta dopadu (px)</t>
+          <t>slider|aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
         </is>
       </c>
     </row>
@@ -4200,32 +4200,32 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
+          <t>PEVNE TELA (nikto cez nikoho neprejde)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>0.7</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>Casovanie zasahu v animacii.</t>
+          <t>Zapne pevne nohy postav; nikto cez nikoho neprejde.</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>slider|kedy v animacii uderu zasah plati (0 = hned, 1 = na konci)</t>
+          <t>switch|PEVNE TELA (nikto cez nikoho neprejde)</t>
         </is>
       </c>
     </row>
@@ -4247,17 +4247,17 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
+          <t>pevne telo: hlbka nohy (px; 54 = cele telo)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>0.72</t>
+          <t>30.0</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>Vyska zasiahnutelnej casti nepriatela.</t>
+          <t>Hlbka pevneho tela (odladene 30).</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -4267,7 +4267,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>slider|aky vysoky kus tela nepriatela sa da trafit (0-1)</t>
+          <t>slider|pevne telo: hlbka nohy (px; 54 = cele telo)</t>
         </is>
       </c>
     </row>
@@ -4284,32 +4284,32 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>switch</t>
+          <t>slider</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>PEVNE TELA (nikto cez nikoho neprejde)</t>
+          <t>pevne telo: sirka nohy (px)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>60.0</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>Zapne pevne nohy postav; nikto cez nikoho neprejde.</t>
+          <t>Sirka pevneho tela (odladene 60).</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>switch|PEVNE TELA (nikto cez nikoho neprejde)</t>
+          <t>slider|pevne telo: sirka nohy (px)</t>
         </is>
       </c>
     </row>
@@ -4331,17 +4331,17 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>pevne telo: hlbka nohy (px; 54 = cele telo)</t>
+          <t>ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>30.0</t>
+          <t>46.0</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>Hlbka pevneho tela (odladene 30).</t>
+          <t>Stary mak odtlacania; funguje len ked su PEVNE TELA vypnute.</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -4351,7 +4351,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>slider|pevne telo: hlbka nohy (px; 54 = cele telo)</t>
+          <t>slider|ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
         </is>
       </c>
     </row>
@@ -4363,7 +4363,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>ODHODENIE PO ZASAHU</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4373,27 +4373,27 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>pevne telo: sirka nohy (px)</t>
+          <t>bezec odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>60.0</t>
+          <t>90.0</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>Sirka pevneho tela (odladene 60).</t>
+          <t>Dlzka odhodenia hrdinu po zasahu bezca.</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>slider|pevne telo: sirka nohy (px)</t>
+          <t>slider|bezec odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -4405,7 +4405,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>NEPRIATELIA</t>
+          <t>ODHODENIE PO ZASAHU</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -4415,27 +4415,27 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
+          <t>strela strelca odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>46.0</t>
+          <t>35.0</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>Stary mak odtlacania; funguje len ked su PEVNE TELA vypnute.</t>
+          <t>Dlzka odhodenia hrdinu po zasahu strely.</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>A</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>slider|ako daleko od seba sa nepriatelia odtlacaju (px; len bez pevnych tiel)</t>
+          <t>slider|strela strelca odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -4457,17 +4457,17 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>bezec odhodi hrdinu (px)</t>
+          <t>sekera odhodi nepriatela (px)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>90.0</t>
+          <t>70.0</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu po zasahu bezca.</t>
+          <t>Dlzka odhodenia nepriatela po zasahu sekery.</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -4477,7 +4477,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>slider|bezec odhodi hrdinu (px)</t>
+          <t>slider|sekera odhodi nepriatela (px)</t>
         </is>
       </c>
     </row>
@@ -4499,17 +4499,17 @@
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>strela strelca odhodi hrdinu (px)</t>
+          <t>vybuch kotla odhodi hrdinu (px)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>35.0</t>
+          <t>140.0</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu po zasahu strely.</t>
+          <t>Dlzka odhodenia hrdinu pri vybuchu kotla.</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -4519,7 +4519,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>slider|strela strelca odhodi hrdinu (px)</t>
+          <t>slider|vybuch kotla odhodi hrdinu (px)</t>
         </is>
       </c>
     </row>
@@ -4541,27 +4541,27 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>sekera odhodi nepriatela (px)</t>
+          <t>odhodenie: ako dlho trva (s)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>0.4</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia nepriatela po zasahu sekery.</t>
+          <t>Trvanie odhodenia (odladene 0,4).</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>slider|sekera odhodi nepriatela (px)</t>
+          <t>slider|odhodenie: ako dlho trva (s)</t>
         </is>
       </c>
     </row>
@@ -4573,7 +4573,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>SRDIECKA A TIENE</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -4583,17 +4583,17 @@
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>vybuch kotla odhodi hrdinu (px)</t>
+          <t>srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>140.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>Dlzka odhodenia hrdinu pri vybuchu kotla.</t>
+          <t>Zivoty nad postavami.</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -4603,7 +4603,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>slider|vybuch kotla odhodi hrdinu (px)</t>
+          <t>slider|srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
         </is>
       </c>
     </row>
@@ -4615,7 +4615,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>ODHODENIE PO ZASAHU</t>
+          <t>SRDIECKA A TIENE</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -4625,17 +4625,17 @@
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>odhodenie: ako dlho trva (s)</t>
+          <t>tien pod postavami: sila (0 = vypnuty)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>0.4</t>
+          <t>0.3</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>Trvanie odhodenia (odladene 0,4).</t>
+          <t>Sila tiena (odladene 0,3).</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -4645,7 +4645,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>slider|odhodenie: ako dlho trva (s)</t>
+          <t>slider|tien pod postavami: sila (0 = vypnuty)</t>
         </is>
       </c>
     </row>
@@ -4667,27 +4667,27 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+          <t>tien pod postavami: velkost (x)</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>1.0</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Zivoty nad postavami.</t>
+          <t>Velkost tiena (odladene 1).</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>slider|srdiecka nad postavami: 0 vypnute, 1 hrdina + ranene, 2 vsetci</t>
+          <t>slider|tien pod postavami: velkost (x)</t>
         </is>
       </c>
     </row>
@@ -4699,7 +4699,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>ZONA PRE LAVY PALEC</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -4709,17 +4709,17 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>tien pod postavami: sila (0 = vypnuty)</t>
+          <t>sirka</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>Sila tiena (odladene 0,3).</t>
+          <t>Sirka zony pre lavy palec.</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -4729,7 +4729,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>slider|tien pod postavami: sila (0 = vypnuty)</t>
+          <t>slider|sirka</t>
         </is>
       </c>
     </row>
@@ -4741,7 +4741,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>SRDIECKA A TIENE</t>
+          <t>ZONA PRE LAVY PALEC</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -4751,17 +4751,17 @@
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>tien pod postavami: velkost (x)</t>
+          <t>kolko zospodu patri miereniu</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>1.0</t>
+          <t>0.16</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>Velkost tiena (odladene 1).</t>
+          <t>Spodna cast zony patri miereniu.</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -4771,7 +4771,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>slider|tien pod postavami: velkost (x)</t>
+          <t>slider|kolko zospodu patri miereniu</t>
         </is>
       </c>
     </row>
@@ -4788,22 +4788,22 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>sirka</t>
+          <t>MIERIT OD POSTAVY</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>Sirka zony pre lavy palec.</t>
+          <t>Mierenie zacina od postavy.</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -4813,7 +4813,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>slider|sirka</t>
+          <t>switch|MIERIT OD POSTAVY</t>
         </is>
       </c>
     </row>
@@ -4830,22 +4830,22 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>slider</t>
+          <t>switch</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>kolko zospodu patri miereniu</t>
+          <t>VOLNY POHYB (bez skoku)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>0.16</t>
+          <t>ZAP</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>Spodna cast zony patri miereniu.</t>
+          <t>Hrdina nechodi skokom k prstu.</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -4855,7 +4855,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>slider|kolko zospodu patri miereniu</t>
+          <t>switch|VOLNY POHYB (bez skoku)</t>
         </is>
       </c>
     </row>
@@ -4877,17 +4877,17 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>MIERIT OD POSTAVY</t>
+          <t>POHYB KOPIRUJE PALEC</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>ZAP</t>
+          <t>VYP</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>Mierenie zacina od postavy.</t>
+          <t>Hrdina kopiruje pohyb palca.</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -4897,97 +4897,13 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>switch|MIERIT OD POSTAVY</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t>S106</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>ZONA PRE LAVY PALEC</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>switch</t>
-        </is>
-      </c>
-      <c r="D107" s="2" t="inlineStr">
-        <is>
-          <t>VOLNY POHYB (bez skoku)</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>ZAP</t>
-        </is>
-      </c>
-      <c r="F107" s="2" t="inlineStr">
-        <is>
-          <t>Hrdina nechodi skokom k prstu.</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H107" t="inlineStr">
-        <is>
-          <t>switch|VOLNY POHYB (bez skoku)</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t>S107</t>
-        </is>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>ZONA PRE LAVY PALEC</t>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>switch</t>
-        </is>
-      </c>
-      <c r="D108" s="2" t="inlineStr">
-        <is>
-          <t>POHYB KOPIRUJE PALEC</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>VYP</t>
-        </is>
-      </c>
-      <c r="F108" s="2" t="inlineStr">
-        <is>
-          <t>Hrdina kopiruje pohyb palca.</t>
-        </is>
-      </c>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
           <t>switch|POHYB KOPIRUJE PALEC</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G108"/>
-  <conditionalFormatting sqref="G2:G108">
+  <autoFilter ref="A1:G106"/>
+  <conditionalFormatting sqref="G2:G106">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"A"</formula>
     </cfRule>
@@ -4996,7 +4912,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G108" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G106" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"A,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>